<commit_message>
Primera corrección sobre nuestro modelo de dominio ConjuntosResidenciales TipoZonaInmueble, TipoInmueble y UnidadTiempoUso
</commit_message>
<xml_diff>
--- a/Doo-Doc/Nueva Version Victus/Modelos de Dominio Enriquecidos/Modelo De Dominio Enriquecido Agendas.xlsx
+++ b/Doo-Doc/Nueva Version Victus/Modelos de Dominio Enriquecidos/Modelo De Dominio Enriquecido Agendas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Music\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\DOO 2024 BD\DOO\victus-doc\Doo-Doc\Nueva Version Victus\Modelos de Dominio Enriquecidos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B8382B7-8CA5-45B7-8ED0-384119DBB487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA236762-3ED3-439A-B8E7-742C55D62F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="2" activeTab="4" xr2:uid="{9E75F319-B909-453D-9AFC-FA9C5B40B20E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="4" xr2:uid="{9E75F319-B909-453D-9AFC-FA9C5B40B20E}"/>
   </bookViews>
   <sheets>
     <sheet name="Valores" sheetId="1" r:id="rId1"/>
@@ -2733,6 +2733,51 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2754,38 +2799,173 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2793,45 +2973,15 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2840,156 +2990,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="27" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3092,8 +3092,8 @@
       <sheetName val="Inmueble"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
       <sheetData sheetId="2">
         <row r="4">
           <cell r="A4" t="str">
@@ -3104,11 +3104,11 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -3432,19 +3432,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AC31824-1358-4896-8FEC-CA18F2D1F29C}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="50" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B1" s="66"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -3452,7 +3452,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
@@ -3460,7 +3460,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
@@ -3468,52 +3468,52 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>15</v>
       </c>
@@ -3529,7 +3529,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{270AC7B1-5317-4DF0-8E73-05A502D22732}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3539,26 +3539,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6DC33F5-6024-4ECE-8864-A6190D431B22}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="56.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="11.42578125" style="8"/>
+    <col min="1" max="1" width="21.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="56.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="11.44140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="52" t="s">
+      <c r="B1" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="52"/>
-      <c r="D1" s="53"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C1" s="67"/>
+      <c r="D1" s="68"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>17</v>
       </c>
@@ -3572,7 +3572,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
         <v>20</v>
       </c>
@@ -3582,12 +3582,12 @@
       <c r="C3" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="54" t="str">
+      <c r="D3" s="69" t="str">
         <f>$B$1</f>
         <v>Agendas</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>21</v>
       </c>
@@ -3597,9 +3597,9 @@
       <c r="C4" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="55"/>
-    </row>
-    <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="D4" s="70"/>
+    </row>
+    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
         <v>22</v>
       </c>
@@ -3609,7 +3609,7 @@
       <c r="C5" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="56"/>
+      <c r="D5" s="71"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3628,103 +3628,103 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0BC2B36-176F-457B-9E5A-2C1354FBA2A7}">
   <dimension ref="A1:U27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" style="8" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="61.28515625" style="8" customWidth="1"/>
-    <col min="10" max="10" width="79.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" style="8" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="61.33203125" style="8" customWidth="1"/>
+    <col min="10" max="10" width="79.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.88671875" style="8" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="25" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="94.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="39.7109375" style="8" customWidth="1"/>
-    <col min="19" max="19" width="46.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="32.42578125" style="8" customWidth="1"/>
-    <col min="21" max="21" width="25.42578125" style="8" customWidth="1"/>
-    <col min="22" max="22" width="52.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="11.42578125" style="8"/>
+    <col min="17" max="17" width="94.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="39.6640625" style="8" customWidth="1"/>
+    <col min="19" max="19" width="46.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="32.44140625" style="8" customWidth="1"/>
+    <col min="21" max="21" width="25.44140625" style="8" customWidth="1"/>
+    <col min="22" max="22" width="52.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="11.44140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A1" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
-      <c r="H1" s="75"/>
-      <c r="I1" s="75"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
+      <c r="D1" s="121"/>
+      <c r="E1" s="121"/>
+      <c r="F1" s="121"/>
+      <c r="G1" s="121"/>
+      <c r="H1" s="121"/>
+      <c r="I1" s="121"/>
+      <c r="J1" s="121"/>
+      <c r="K1" s="121"/>
+      <c r="L1" s="121"/>
+      <c r="M1" s="121"/>
+      <c r="N1" s="121"/>
+      <c r="O1" s="121"/>
+      <c r="P1" s="121"/>
+      <c r="Q1" s="121"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="76" t="str">
+      <c r="B2" s="122" t="str">
         <f>'[1]Listado Objetos Dominio'!A4</f>
         <v>ZonaComun</v>
       </c>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="76"/>
-      <c r="M2" s="76"/>
-      <c r="N2" s="76"/>
-      <c r="O2" s="76"/>
-      <c r="P2" s="76"/>
-      <c r="Q2" s="76"/>
-    </row>
-    <row r="3" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="122"/>
+      <c r="D2" s="122"/>
+      <c r="E2" s="122"/>
+      <c r="F2" s="122"/>
+      <c r="G2" s="122"/>
+      <c r="H2" s="122"/>
+      <c r="I2" s="122"/>
+      <c r="J2" s="122"/>
+      <c r="K2" s="122"/>
+      <c r="L2" s="122"/>
+      <c r="M2" s="122"/>
+      <c r="N2" s="122"/>
+      <c r="O2" s="122"/>
+      <c r="P2" s="122"/>
+      <c r="Q2" s="122"/>
+    </row>
+    <row r="3" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="77" t="str">
+      <c r="B3" s="123" t="str">
         <f>'[1]Listado Objetos Dominio'!B4</f>
         <v>Objeto de dominio que representa a cada una de las zonas comunes que se encuentran dentro de un conjunto residencial para que los residentes puedan reservar esos espacios y poder usarlos.</v>
       </c>
-      <c r="C3" s="77"/>
-      <c r="D3" s="77"/>
-      <c r="E3" s="77"/>
-      <c r="F3" s="77"/>
-      <c r="G3" s="77"/>
-      <c r="H3" s="77"/>
-      <c r="I3" s="77"/>
-      <c r="J3" s="77"/>
-      <c r="K3" s="77"/>
-      <c r="L3" s="77"/>
-      <c r="M3" s="77"/>
-      <c r="N3" s="77"/>
-      <c r="O3" s="77"/>
-      <c r="P3" s="77"/>
-      <c r="Q3" s="77"/>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="C3" s="123"/>
+      <c r="D3" s="123"/>
+      <c r="E3" s="123"/>
+      <c r="F3" s="123"/>
+      <c r="G3" s="123"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
+      <c r="L3" s="123"/>
+      <c r="M3" s="123"/>
+      <c r="N3" s="123"/>
+      <c r="O3" s="123"/>
+      <c r="P3" s="123"/>
+      <c r="Q3" s="123"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>30</v>
       </c>
@@ -3776,24 +3776,24 @@
       <c r="Q4" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="R4" s="126" t="str">
+      <c r="R4" s="57" t="str">
         <f>A21</f>
         <v>Registrar</v>
       </c>
-      <c r="S4" s="127" t="str">
+      <c r="S4" s="58" t="str">
         <f>A25</f>
         <v>Buscar</v>
       </c>
-      <c r="T4" s="128" t="str">
+      <c r="T4" s="59" t="str">
         <f>A26</f>
         <v>Modificar</v>
       </c>
-      <c r="U4" s="129" t="str">
+      <c r="U4" s="60" t="str">
         <f>A27</f>
         <v>Eliminar</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
         <v>46</v>
       </c>
@@ -3833,7 +3833,7 @@
       <c r="Q5" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="R5" s="130" t="s">
+      <c r="R5" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S5" s="23" t="s">
@@ -3846,7 +3846,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A6" s="26" t="s">
         <v>50</v>
       </c>
@@ -3888,7 +3888,7 @@
       <c r="Q6" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="R6" s="130" t="s">
+      <c r="R6" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S6" s="23" t="s">
@@ -3901,7 +3901,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
         <v>66</v>
       </c>
@@ -3943,7 +3943,7 @@
       <c r="Q7" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="R7" s="130" t="s">
+      <c r="R7" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S7" s="23" t="s">
@@ -3956,7 +3956,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8" s="26" t="s">
         <v>87</v>
       </c>
@@ -3992,7 +3992,7 @@
       <c r="Q8" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="R8" s="130" t="s">
+      <c r="R8" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S8" s="23" t="s">
@@ -4005,7 +4005,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>88</v>
       </c>
@@ -4043,7 +4043,7 @@
       <c r="Q9" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="R9" s="130" t="s">
+      <c r="R9" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S9" s="23" t="s">
@@ -4056,7 +4056,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="26" t="s">
         <v>89</v>
       </c>
@@ -4092,7 +4092,7 @@
       <c r="Q10" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="R10" s="130" t="s">
+      <c r="R10" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S10" s="23" t="s">
@@ -4105,7 +4105,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A11" s="26" t="s">
         <v>67</v>
       </c>
@@ -4147,7 +4147,7 @@
       <c r="Q11" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="R11" s="130" t="s">
+      <c r="R11" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S11" s="23" t="s">
@@ -4160,7 +4160,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="45" t="s">
         <v>68</v>
       </c>
@@ -4194,7 +4194,7 @@
       <c r="Q12" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="R12" s="130" t="s">
+      <c r="R12" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S12" s="37" t="s">
@@ -4207,15 +4207,15 @@
         <v>140</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="72" t="s">
+    <row r="13" spans="1:21" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="14" spans="1:21" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="118" t="s">
         <v>98</v>
       </c>
-      <c r="B14" s="73"/>
-      <c r="C14" s="74"/>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B14" s="119"/>
+      <c r="C14" s="120"/>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" s="27" t="s">
         <v>53</v>
       </c>
@@ -4226,66 +4226,66 @@
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="131" t="s">
+    <row r="16" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="124" t="s">
         <v>99</v>
       </c>
-      <c r="B16" s="80" t="s">
+      <c r="B16" s="126" t="s">
         <v>100</v>
       </c>
       <c r="C16" s="30" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="132"/>
-      <c r="B17" s="81"/>
+    <row r="17" spans="1:19" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="125"/>
+      <c r="B17" s="127"/>
       <c r="C17" s="31" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A19" s="68" t="s">
+    <row r="18" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A19" s="128" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="57"/>
-      <c r="C19" s="57" t="s">
+      <c r="B19" s="115"/>
+      <c r="C19" s="115" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="57"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="57"/>
-      <c r="G19" s="57"/>
-      <c r="H19" s="57" t="s">
+      <c r="D19" s="115"/>
+      <c r="E19" s="115"/>
+      <c r="F19" s="115"/>
+      <c r="G19" s="115"/>
+      <c r="H19" s="115" t="s">
         <v>56</v>
       </c>
-      <c r="I19" s="57"/>
-      <c r="J19" s="57"/>
-      <c r="K19" s="57" t="s">
+      <c r="I19" s="115"/>
+      <c r="J19" s="115"/>
+      <c r="K19" s="115" t="s">
         <v>57</v>
       </c>
-      <c r="L19" s="57"/>
-      <c r="M19" s="57"/>
-      <c r="N19" s="57"/>
-      <c r="O19" s="57"/>
-      <c r="P19" s="57" t="s">
+      <c r="L19" s="115"/>
+      <c r="M19" s="115"/>
+      <c r="N19" s="115"/>
+      <c r="O19" s="115"/>
+      <c r="P19" s="115" t="s">
         <v>58</v>
       </c>
-      <c r="Q19" s="57"/>
-      <c r="R19" s="57" t="s">
+      <c r="Q19" s="115"/>
+      <c r="R19" s="115" t="s">
         <v>59</v>
       </c>
-      <c r="S19" s="71"/>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A20" s="69"/>
-      <c r="B20" s="70"/>
-      <c r="C20" s="70"/>
-      <c r="D20" s="70"/>
-      <c r="E20" s="70"/>
-      <c r="F20" s="70"/>
-      <c r="G20" s="70"/>
+      <c r="S19" s="116"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A20" s="129"/>
+      <c r="B20" s="117"/>
+      <c r="C20" s="117"/>
+      <c r="D20" s="117"/>
+      <c r="E20" s="117"/>
+      <c r="F20" s="117"/>
+      <c r="G20" s="117"/>
       <c r="H20" s="32" t="s">
         <v>60</v>
       </c>
@@ -4298,12 +4298,12 @@
       <c r="K20" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="L20" s="70" t="s">
+      <c r="L20" s="117" t="s">
         <v>2</v>
       </c>
-      <c r="M20" s="70"/>
-      <c r="N20" s="70"/>
-      <c r="O20" s="70"/>
+      <c r="M20" s="117"/>
+      <c r="N20" s="117"/>
+      <c r="O20" s="117"/>
       <c r="P20" s="32" t="s">
         <v>62</v>
       </c>
@@ -4317,32 +4317,32 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="105" x14ac:dyDescent="0.25">
-      <c r="A21" s="86" t="s">
+    <row r="21" spans="1:19" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="103" t="s">
         <v>119</v>
       </c>
-      <c r="B21" s="87"/>
-      <c r="C21" s="88" t="s">
+      <c r="B21" s="104"/>
+      <c r="C21" s="84" t="s">
         <v>120</v>
       </c>
-      <c r="D21" s="89"/>
-      <c r="E21" s="89"/>
-      <c r="F21" s="89"/>
-      <c r="G21" s="90"/>
-      <c r="H21" s="54" t="s">
+      <c r="D21" s="85"/>
+      <c r="E21" s="85"/>
+      <c r="F21" s="85"/>
+      <c r="G21" s="86"/>
+      <c r="H21" s="69" t="s">
         <v>144</v>
       </c>
-      <c r="I21" s="91" t="s">
+      <c r="I21" s="109" t="s">
         <v>20</v>
       </c>
-      <c r="J21" s="92" t="s">
+      <c r="J21" s="112" t="s">
         <v>145</v>
       </c>
-      <c r="K21" s="93"/>
-      <c r="L21" s="88"/>
-      <c r="M21" s="89"/>
-      <c r="N21" s="89"/>
-      <c r="O21" s="90"/>
+      <c r="K21" s="50"/>
+      <c r="L21" s="84"/>
+      <c r="M21" s="85"/>
+      <c r="N21" s="85"/>
+      <c r="O21" s="86"/>
       <c r="P21" s="14" t="s">
         <v>146</v>
       </c>
@@ -4352,26 +4352,26 @@
       <c r="R21" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="S21" s="94" t="s">
+      <c r="S21" s="51" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="75" x14ac:dyDescent="0.25">
-      <c r="A22" s="95"/>
-      <c r="B22" s="96"/>
-      <c r="C22" s="97"/>
-      <c r="D22" s="98"/>
-      <c r="E22" s="98"/>
-      <c r="F22" s="98"/>
-      <c r="G22" s="99"/>
-      <c r="H22" s="55"/>
-      <c r="I22" s="100"/>
-      <c r="J22" s="101"/>
-      <c r="K22" s="102"/>
-      <c r="L22" s="97"/>
-      <c r="M22" s="98"/>
-      <c r="N22" s="98"/>
-      <c r="O22" s="99"/>
+    <row r="22" spans="1:19" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="105"/>
+      <c r="B22" s="106"/>
+      <c r="C22" s="87"/>
+      <c r="D22" s="88"/>
+      <c r="E22" s="88"/>
+      <c r="F22" s="88"/>
+      <c r="G22" s="89"/>
+      <c r="H22" s="70"/>
+      <c r="I22" s="110"/>
+      <c r="J22" s="113"/>
+      <c r="K22" s="52"/>
+      <c r="L22" s="87"/>
+      <c r="M22" s="88"/>
+      <c r="N22" s="88"/>
+      <c r="O22" s="89"/>
       <c r="P22" s="14" t="s">
         <v>148</v>
       </c>
@@ -4381,26 +4381,26 @@
       <c r="R22" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="S22" s="94" t="s">
+      <c r="S22" s="51" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A23" s="95"/>
-      <c r="B23" s="96"/>
-      <c r="C23" s="97"/>
-      <c r="D23" s="98"/>
-      <c r="E23" s="98"/>
-      <c r="F23" s="98"/>
-      <c r="G23" s="99"/>
-      <c r="H23" s="55"/>
-      <c r="I23" s="100"/>
-      <c r="J23" s="101"/>
-      <c r="K23" s="102"/>
-      <c r="L23" s="97"/>
-      <c r="M23" s="98"/>
-      <c r="N23" s="98"/>
-      <c r="O23" s="99"/>
+    <row r="23" spans="1:19" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="105"/>
+      <c r="B23" s="106"/>
+      <c r="C23" s="87"/>
+      <c r="D23" s="88"/>
+      <c r="E23" s="88"/>
+      <c r="F23" s="88"/>
+      <c r="G23" s="89"/>
+      <c r="H23" s="70"/>
+      <c r="I23" s="110"/>
+      <c r="J23" s="113"/>
+      <c r="K23" s="52"/>
+      <c r="L23" s="87"/>
+      <c r="M23" s="88"/>
+      <c r="N23" s="88"/>
+      <c r="O23" s="89"/>
       <c r="P23" s="14" t="s">
         <v>152</v>
       </c>
@@ -4410,26 +4410,26 @@
       <c r="R23" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="S23" s="94" t="s">
+      <c r="S23" s="51" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="75" x14ac:dyDescent="0.25">
-      <c r="A24" s="103"/>
-      <c r="B24" s="104"/>
-      <c r="C24" s="105"/>
-      <c r="D24" s="106"/>
-      <c r="E24" s="106"/>
-      <c r="F24" s="106"/>
-      <c r="G24" s="107"/>
-      <c r="H24" s="56"/>
-      <c r="I24" s="108"/>
-      <c r="J24" s="109"/>
-      <c r="K24" s="110"/>
-      <c r="L24" s="105"/>
-      <c r="M24" s="106"/>
-      <c r="N24" s="106"/>
-      <c r="O24" s="107"/>
+    <row r="24" spans="1:19" ht="72" x14ac:dyDescent="0.3">
+      <c r="A24" s="107"/>
+      <c r="B24" s="108"/>
+      <c r="C24" s="90"/>
+      <c r="D24" s="91"/>
+      <c r="E24" s="91"/>
+      <c r="F24" s="91"/>
+      <c r="G24" s="92"/>
+      <c r="H24" s="71"/>
+      <c r="I24" s="111"/>
+      <c r="J24" s="114"/>
+      <c r="K24" s="53"/>
+      <c r="L24" s="90"/>
+      <c r="M24" s="91"/>
+      <c r="N24" s="91"/>
+      <c r="O24" s="92"/>
       <c r="P24" s="14" t="s">
         <v>156</v>
       </c>
@@ -4439,22 +4439,22 @@
       <c r="R24" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="S24" s="94" t="s">
+      <c r="S24" s="51" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="105" x14ac:dyDescent="0.25">
-      <c r="A25" s="61" t="s">
+    <row r="25" spans="1:19" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A25" s="93" t="s">
         <v>123</v>
       </c>
-      <c r="B25" s="62"/>
-      <c r="C25" s="63" t="s">
+      <c r="B25" s="94"/>
+      <c r="C25" s="95" t="s">
         <v>160</v>
       </c>
-      <c r="D25" s="63"/>
-      <c r="E25" s="63"/>
-      <c r="F25" s="63"/>
-      <c r="G25" s="63"/>
+      <c r="D25" s="95"/>
+      <c r="E25" s="95"/>
+      <c r="F25" s="95"/>
+      <c r="G25" s="95"/>
       <c r="H25" s="36" t="s">
         <v>144</v>
       </c>
@@ -4467,12 +4467,12 @@
       <c r="K25" s="49" t="s">
         <v>124</v>
       </c>
-      <c r="L25" s="64" t="s">
+      <c r="L25" s="96" t="s">
         <v>125</v>
       </c>
-      <c r="M25" s="64"/>
-      <c r="N25" s="64"/>
-      <c r="O25" s="64"/>
+      <c r="M25" s="96"/>
+      <c r="N25" s="96"/>
+      <c r="O25" s="96"/>
       <c r="P25" s="23" t="s">
         <v>162</v>
       </c>
@@ -4482,22 +4482,22 @@
       <c r="R25" s="37" t="s">
         <v>121</v>
       </c>
-      <c r="S25" s="111" t="s">
+      <c r="S25" s="54" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A26" s="65" t="s">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A26" s="97" t="s">
         <v>127</v>
       </c>
-      <c r="B26" s="66"/>
-      <c r="C26" s="67" t="s">
+      <c r="B26" s="98"/>
+      <c r="C26" s="99" t="s">
         <v>128</v>
       </c>
-      <c r="D26" s="67"/>
-      <c r="E26" s="67"/>
-      <c r="F26" s="67"/>
-      <c r="G26" s="67"/>
+      <c r="D26" s="99"/>
+      <c r="E26" s="99"/>
+      <c r="F26" s="99"/>
+      <c r="G26" s="99"/>
       <c r="H26" s="39" t="s">
         <v>144</v>
       </c>
@@ -4508,75 +4508,56 @@
         <v>163</v>
       </c>
       <c r="K26" s="41"/>
-      <c r="L26" s="112"/>
-      <c r="M26" s="113"/>
-      <c r="N26" s="113"/>
-      <c r="O26" s="114"/>
-      <c r="P26" s="115" t="s">
+      <c r="L26" s="100"/>
+      <c r="M26" s="101"/>
+      <c r="N26" s="101"/>
+      <c r="O26" s="102"/>
+      <c r="P26" s="72" t="s">
         <v>129</v>
       </c>
-      <c r="Q26" s="116" t="s">
+      <c r="Q26" s="74" t="s">
         <v>130</v>
       </c>
-      <c r="R26" s="116" t="s">
+      <c r="R26" s="74" t="s">
         <v>131</v>
       </c>
-      <c r="S26" s="117" t="s">
+      <c r="S26" s="76" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A27" s="58" t="s">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A27" s="78" t="s">
         <v>133</v>
       </c>
-      <c r="B27" s="59"/>
-      <c r="C27" s="60" t="s">
+      <c r="B27" s="79"/>
+      <c r="C27" s="80" t="s">
         <v>134</v>
       </c>
-      <c r="D27" s="60"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="60"/>
-      <c r="G27" s="60"/>
-      <c r="H27" s="118" t="s">
+      <c r="D27" s="80"/>
+      <c r="E27" s="80"/>
+      <c r="F27" s="80"/>
+      <c r="G27" s="80"/>
+      <c r="H27" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="I27" s="119" t="s">
+      <c r="I27" s="56" t="s">
         <v>9</v>
       </c>
       <c r="J27" s="42" t="s">
         <v>164</v>
       </c>
       <c r="K27" s="43"/>
-      <c r="L27" s="120"/>
-      <c r="M27" s="121"/>
-      <c r="N27" s="121"/>
-      <c r="O27" s="122"/>
-      <c r="P27" s="123"/>
-      <c r="Q27" s="124"/>
-      <c r="R27" s="124"/>
-      <c r="S27" s="125"/>
+      <c r="L27" s="81"/>
+      <c r="M27" s="82"/>
+      <c r="N27" s="82"/>
+      <c r="O27" s="83"/>
+      <c r="P27" s="73"/>
+      <c r="Q27" s="75"/>
+      <c r="R27" s="75"/>
+      <c r="S27" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="P26:P27"/>
-    <mergeCell ref="Q26:Q27"/>
-    <mergeCell ref="R26:R27"/>
-    <mergeCell ref="S26:S27"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="L27:O27"/>
-    <mergeCell ref="L21:O24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="L25:O25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="L26:O26"/>
-    <mergeCell ref="A21:B24"/>
-    <mergeCell ref="C21:G24"/>
-    <mergeCell ref="H21:H24"/>
-    <mergeCell ref="I21:I24"/>
-    <mergeCell ref="J21:J24"/>
     <mergeCell ref="P19:Q19"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="L20:O20"/>
@@ -4590,6 +4571,25 @@
     <mergeCell ref="A19:B20"/>
     <mergeCell ref="C19:G20"/>
     <mergeCell ref="H19:J19"/>
+    <mergeCell ref="L21:O24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="L25:O25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="L26:O26"/>
+    <mergeCell ref="A21:B24"/>
+    <mergeCell ref="C21:G24"/>
+    <mergeCell ref="H21:H24"/>
+    <mergeCell ref="I21:I24"/>
+    <mergeCell ref="J21:J24"/>
+    <mergeCell ref="P26:P27"/>
+    <mergeCell ref="Q26:Q27"/>
+    <mergeCell ref="R26:R27"/>
+    <mergeCell ref="S26:S27"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="L27:O27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de Dominio'!A1" display="Volver al inicio" xr:uid="{86A492AF-8702-4148-85C2-41FF6CA10413}"/>
@@ -4618,103 +4618,103 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{037CC029-DC44-4605-90F4-CA51C57B9385}">
   <dimension ref="A1:U28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" style="8" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="61.28515625" style="8" customWidth="1"/>
-    <col min="10" max="10" width="79.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" style="8" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="61.33203125" style="8" customWidth="1"/>
+    <col min="10" max="10" width="79.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.88671875" style="8" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="25" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="94.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="43.5703125" style="8" customWidth="1"/>
-    <col min="19" max="19" width="46.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="50.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="66.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="52.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="11.42578125" style="8"/>
+    <col min="17" max="17" width="94.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="43.5546875" style="8" customWidth="1"/>
+    <col min="19" max="19" width="46.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="50.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="66.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="52.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="11.44140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A1" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
-      <c r="H1" s="75"/>
-      <c r="I1" s="75"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
+      <c r="D1" s="121"/>
+      <c r="E1" s="121"/>
+      <c r="F1" s="121"/>
+      <c r="G1" s="121"/>
+      <c r="H1" s="121"/>
+      <c r="I1" s="121"/>
+      <c r="J1" s="121"/>
+      <c r="K1" s="121"/>
+      <c r="L1" s="121"/>
+      <c r="M1" s="121"/>
+      <c r="N1" s="121"/>
+      <c r="O1" s="121"/>
+      <c r="P1" s="121"/>
+      <c r="Q1" s="121"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="76" t="str">
+      <c r="B2" s="122" t="str">
         <f>'Listado Objetos de Dominio'!A4</f>
         <v>Agenda</v>
       </c>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="76"/>
-      <c r="M2" s="76"/>
-      <c r="N2" s="76"/>
-      <c r="O2" s="76"/>
-      <c r="P2" s="76"/>
-      <c r="Q2" s="76"/>
-    </row>
-    <row r="3" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="122"/>
+      <c r="D2" s="122"/>
+      <c r="E2" s="122"/>
+      <c r="F2" s="122"/>
+      <c r="G2" s="122"/>
+      <c r="H2" s="122"/>
+      <c r="I2" s="122"/>
+      <c r="J2" s="122"/>
+      <c r="K2" s="122"/>
+      <c r="L2" s="122"/>
+      <c r="M2" s="122"/>
+      <c r="N2" s="122"/>
+      <c r="O2" s="122"/>
+      <c r="P2" s="122"/>
+      <c r="Q2" s="122"/>
+    </row>
+    <row r="3" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="77" t="str">
+      <c r="B3" s="123" t="str">
         <f>'Listado Objetos de Dominio'!B4</f>
         <v>Objeto de dominio que representaa cada una de las agendas que dónde el residente podrá reservar.</v>
       </c>
-      <c r="C3" s="77"/>
-      <c r="D3" s="77"/>
-      <c r="E3" s="77"/>
-      <c r="F3" s="77"/>
-      <c r="G3" s="77"/>
-      <c r="H3" s="77"/>
-      <c r="I3" s="77"/>
-      <c r="J3" s="77"/>
-      <c r="K3" s="77"/>
-      <c r="L3" s="77"/>
-      <c r="M3" s="77"/>
-      <c r="N3" s="77"/>
-      <c r="O3" s="77"/>
-      <c r="P3" s="77"/>
-      <c r="Q3" s="77"/>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="C3" s="123"/>
+      <c r="D3" s="123"/>
+      <c r="E3" s="123"/>
+      <c r="F3" s="123"/>
+      <c r="G3" s="123"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
+      <c r="L3" s="123"/>
+      <c r="M3" s="123"/>
+      <c r="N3" s="123"/>
+      <c r="O3" s="123"/>
+      <c r="P3" s="123"/>
+      <c r="Q3" s="123"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>30</v>
       </c>
@@ -4766,24 +4766,24 @@
       <c r="Q4" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="R4" s="126" t="str">
+      <c r="R4" s="57" t="str">
         <f>A21</f>
         <v>Registrar</v>
       </c>
-      <c r="S4" s="127" t="str">
+      <c r="S4" s="58" t="str">
         <f>A26</f>
         <v>Buscar</v>
       </c>
-      <c r="T4" s="128" t="str">
+      <c r="T4" s="59" t="str">
         <f>A27</f>
         <v>Modificar</v>
       </c>
-      <c r="U4" s="129" t="str">
+      <c r="U4" s="60" t="str">
         <f>A28</f>
         <v>Eliminar</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
         <v>46</v>
       </c>
@@ -4823,7 +4823,7 @@
       <c r="Q5" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="R5" s="130" t="s">
+      <c r="R5" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S5" s="23" t="s">
@@ -4836,7 +4836,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A6" s="26" t="s">
         <v>50</v>
       </c>
@@ -4878,7 +4878,7 @@
       <c r="Q6" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="R6" s="130" t="s">
+      <c r="R6" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S6" s="23" t="s">
@@ -4891,7 +4891,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
         <v>101</v>
       </c>
@@ -4929,7 +4929,7 @@
       <c r="Q7" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="R7" s="130" t="s">
+      <c r="R7" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S7" s="23" t="s">
@@ -4942,7 +4942,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A8" s="26" t="s">
         <v>69</v>
       </c>
@@ -4978,7 +4978,7 @@
       <c r="Q8" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="R8" s="130" t="s">
+      <c r="R8" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S8" s="23" t="s">
@@ -4991,7 +4991,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>70</v>
       </c>
@@ -5027,7 +5027,7 @@
       <c r="Q9" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="R9" s="130" t="s">
+      <c r="R9" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S9" s="23" t="s">
@@ -5040,7 +5040,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="47" t="s">
         <v>71</v>
       </c>
@@ -5076,7 +5076,7 @@
       <c r="Q10" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="R10" s="130" t="s">
+      <c r="R10" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S10" s="37" t="s">
@@ -5089,15 +5089,15 @@
         <v>140</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="72" t="s">
+    <row r="11" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:21" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="118" t="s">
         <v>98</v>
       </c>
-      <c r="B12" s="73"/>
-      <c r="C12" s="74"/>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B12" s="119"/>
+      <c r="C12" s="120"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" s="27" t="s">
         <v>53</v>
       </c>
@@ -5108,78 +5108,78 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="78" t="s">
+    <row r="14" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="130" t="s">
         <v>82</v>
       </c>
-      <c r="B14" s="80" t="s">
+      <c r="B14" s="126" t="s">
         <v>108</v>
       </c>
-      <c r="C14" s="84" t="s">
+      <c r="C14" s="134" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="82"/>
-      <c r="B15" s="83"/>
-      <c r="C15" s="85"/>
-    </row>
-    <row r="16" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="82"/>
-      <c r="B16" s="83"/>
+    <row r="15" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="131"/>
+      <c r="B15" s="133"/>
+      <c r="C15" s="135"/>
+    </row>
+    <row r="16" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="131"/>
+      <c r="B16" s="133"/>
       <c r="C16" s="30" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="20.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="79"/>
-      <c r="B17" s="81"/>
+    <row r="17" spans="1:19" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="132"/>
+      <c r="B17" s="127"/>
       <c r="C17" s="46" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A19" s="68" t="s">
+    <row r="18" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A19" s="128" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="57"/>
-      <c r="C19" s="57" t="s">
+      <c r="B19" s="115"/>
+      <c r="C19" s="115" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="57"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="57"/>
-      <c r="G19" s="57"/>
-      <c r="H19" s="57" t="s">
+      <c r="D19" s="115"/>
+      <c r="E19" s="115"/>
+      <c r="F19" s="115"/>
+      <c r="G19" s="115"/>
+      <c r="H19" s="115" t="s">
         <v>56</v>
       </c>
-      <c r="I19" s="57"/>
-      <c r="J19" s="57"/>
-      <c r="K19" s="57" t="s">
+      <c r="I19" s="115"/>
+      <c r="J19" s="115"/>
+      <c r="K19" s="115" t="s">
         <v>57</v>
       </c>
-      <c r="L19" s="57"/>
-      <c r="M19" s="57"/>
-      <c r="N19" s="57"/>
-      <c r="O19" s="57"/>
-      <c r="P19" s="57" t="s">
+      <c r="L19" s="115"/>
+      <c r="M19" s="115"/>
+      <c r="N19" s="115"/>
+      <c r="O19" s="115"/>
+      <c r="P19" s="115" t="s">
         <v>58</v>
       </c>
-      <c r="Q19" s="57"/>
-      <c r="R19" s="57" t="s">
+      <c r="Q19" s="115"/>
+      <c r="R19" s="115" t="s">
         <v>59</v>
       </c>
-      <c r="S19" s="71"/>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A20" s="69"/>
-      <c r="B20" s="70"/>
-      <c r="C20" s="70"/>
-      <c r="D20" s="70"/>
-      <c r="E20" s="70"/>
-      <c r="F20" s="70"/>
-      <c r="G20" s="70"/>
+      <c r="S19" s="116"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A20" s="129"/>
+      <c r="B20" s="117"/>
+      <c r="C20" s="117"/>
+      <c r="D20" s="117"/>
+      <c r="E20" s="117"/>
+      <c r="F20" s="117"/>
+      <c r="G20" s="117"/>
       <c r="H20" s="32" t="s">
         <v>60</v>
       </c>
@@ -5192,12 +5192,12 @@
       <c r="K20" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="L20" s="70" t="s">
+      <c r="L20" s="117" t="s">
         <v>2</v>
       </c>
-      <c r="M20" s="70"/>
-      <c r="N20" s="70"/>
-      <c r="O20" s="70"/>
+      <c r="M20" s="117"/>
+      <c r="N20" s="117"/>
+      <c r="O20" s="117"/>
       <c r="P20" s="32" t="s">
         <v>62</v>
       </c>
@@ -5211,35 +5211,35 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="87" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="86" t="s">
+    <row r="21" spans="1:19" ht="87" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="103" t="s">
         <v>119</v>
       </c>
-      <c r="B21" s="87"/>
-      <c r="C21" s="88" t="s">
+      <c r="B21" s="104"/>
+      <c r="C21" s="84" t="s">
         <v>198</v>
       </c>
-      <c r="D21" s="89"/>
-      <c r="E21" s="89"/>
-      <c r="F21" s="89"/>
-      <c r="G21" s="90"/>
-      <c r="H21" s="54" t="str">
+      <c r="D21" s="85"/>
+      <c r="E21" s="85"/>
+      <c r="F21" s="85"/>
+      <c r="G21" s="86"/>
+      <c r="H21" s="69" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosAgenda</v>
       </c>
-      <c r="I21" s="91" t="str">
+      <c r="I21" s="109" t="str">
         <f>B2</f>
         <v>Agenda</v>
       </c>
-      <c r="J21" s="92" t="str">
+      <c r="J21" s="112" t="str">
         <f>_xlfn.CONCAT("Corresponde al objeto que internamente contiene los datos necesarios para crear una nueva ",$B$2,)</f>
         <v>Corresponde al objeto que internamente contiene los datos necesarios para crear una nueva Agenda</v>
       </c>
-      <c r="K21" s="93"/>
-      <c r="L21" s="88"/>
-      <c r="M21" s="89"/>
-      <c r="N21" s="89"/>
-      <c r="O21" s="90"/>
+      <c r="K21" s="50"/>
+      <c r="L21" s="84"/>
+      <c r="M21" s="85"/>
+      <c r="N21" s="85"/>
+      <c r="O21" s="86"/>
       <c r="P21" s="14" t="s">
         <v>187</v>
       </c>
@@ -5249,26 +5249,26 @@
       <c r="R21" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="S21" s="94" t="s">
+      <c r="S21" s="51" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="108.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="95"/>
-      <c r="B22" s="96"/>
-      <c r="C22" s="97"/>
-      <c r="D22" s="98"/>
-      <c r="E22" s="98"/>
-      <c r="F22" s="98"/>
-      <c r="G22" s="99"/>
-      <c r="H22" s="55"/>
-      <c r="I22" s="100"/>
-      <c r="J22" s="101"/>
-      <c r="K22" s="102"/>
-      <c r="L22" s="97"/>
-      <c r="M22" s="98"/>
-      <c r="N22" s="98"/>
-      <c r="O22" s="99"/>
+    <row r="22" spans="1:19" ht="108.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="105"/>
+      <c r="B22" s="106"/>
+      <c r="C22" s="87"/>
+      <c r="D22" s="88"/>
+      <c r="E22" s="88"/>
+      <c r="F22" s="88"/>
+      <c r="G22" s="89"/>
+      <c r="H22" s="70"/>
+      <c r="I22" s="110"/>
+      <c r="J22" s="113"/>
+      <c r="K22" s="52"/>
+      <c r="L22" s="87"/>
+      <c r="M22" s="88"/>
+      <c r="N22" s="88"/>
+      <c r="O22" s="89"/>
       <c r="P22" s="14" t="s">
         <v>188</v>
       </c>
@@ -5278,26 +5278,26 @@
       <c r="R22" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="S22" s="94" t="s">
+      <c r="S22" s="51" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="123.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="95"/>
-      <c r="B23" s="96"/>
-      <c r="C23" s="97"/>
-      <c r="D23" s="98"/>
-      <c r="E23" s="98"/>
-      <c r="F23" s="98"/>
-      <c r="G23" s="99"/>
-      <c r="H23" s="55"/>
-      <c r="I23" s="100"/>
-      <c r="J23" s="101"/>
-      <c r="K23" s="102"/>
-      <c r="L23" s="97"/>
-      <c r="M23" s="98"/>
-      <c r="N23" s="98"/>
-      <c r="O23" s="99"/>
+    <row r="23" spans="1:19" ht="123.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="105"/>
+      <c r="B23" s="106"/>
+      <c r="C23" s="87"/>
+      <c r="D23" s="88"/>
+      <c r="E23" s="88"/>
+      <c r="F23" s="88"/>
+      <c r="G23" s="89"/>
+      <c r="H23" s="70"/>
+      <c r="I23" s="110"/>
+      <c r="J23" s="113"/>
+      <c r="K23" s="52"/>
+      <c r="L23" s="87"/>
+      <c r="M23" s="88"/>
+      <c r="N23" s="88"/>
+      <c r="O23" s="89"/>
       <c r="P23" s="14" t="s">
         <v>189</v>
       </c>
@@ -5307,26 +5307,26 @@
       <c r="R23" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="S23" s="94" t="s">
+      <c r="S23" s="51" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="111" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="95"/>
-      <c r="B24" s="96"/>
-      <c r="C24" s="97"/>
-      <c r="D24" s="98"/>
-      <c r="E24" s="98"/>
-      <c r="F24" s="98"/>
-      <c r="G24" s="99"/>
-      <c r="H24" s="55"/>
-      <c r="I24" s="100"/>
-      <c r="J24" s="101"/>
-      <c r="K24" s="102"/>
-      <c r="L24" s="97"/>
-      <c r="M24" s="98"/>
-      <c r="N24" s="98"/>
-      <c r="O24" s="99"/>
+    <row r="24" spans="1:19" ht="111" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="105"/>
+      <c r="B24" s="106"/>
+      <c r="C24" s="87"/>
+      <c r="D24" s="88"/>
+      <c r="E24" s="88"/>
+      <c r="F24" s="88"/>
+      <c r="G24" s="89"/>
+      <c r="H24" s="70"/>
+      <c r="I24" s="110"/>
+      <c r="J24" s="113"/>
+      <c r="K24" s="52"/>
+      <c r="L24" s="87"/>
+      <c r="M24" s="88"/>
+      <c r="N24" s="88"/>
+      <c r="O24" s="89"/>
       <c r="P24" s="14" t="s">
         <v>190</v>
       </c>
@@ -5336,26 +5336,26 @@
       <c r="R24" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="S24" s="94" t="s">
+      <c r="S24" s="51" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="87.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="103"/>
-      <c r="B25" s="104"/>
-      <c r="C25" s="105"/>
-      <c r="D25" s="106"/>
-      <c r="E25" s="106"/>
-      <c r="F25" s="106"/>
-      <c r="G25" s="107"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="108"/>
-      <c r="J25" s="109"/>
-      <c r="K25" s="110"/>
-      <c r="L25" s="105"/>
-      <c r="M25" s="106"/>
-      <c r="N25" s="106"/>
-      <c r="O25" s="107"/>
+    <row r="25" spans="1:19" ht="87.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="107"/>
+      <c r="B25" s="108"/>
+      <c r="C25" s="90"/>
+      <c r="D25" s="91"/>
+      <c r="E25" s="91"/>
+      <c r="F25" s="91"/>
+      <c r="G25" s="92"/>
+      <c r="H25" s="71"/>
+      <c r="I25" s="111"/>
+      <c r="J25" s="114"/>
+      <c r="K25" s="53"/>
+      <c r="L25" s="90"/>
+      <c r="M25" s="91"/>
+      <c r="N25" s="91"/>
+      <c r="O25" s="92"/>
       <c r="P25" s="14" t="s">
         <v>191</v>
       </c>
@@ -5365,22 +5365,22 @@
       <c r="R25" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="S25" s="94" t="s">
+      <c r="S25" s="51" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="102.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="61" t="s">
+    <row r="26" spans="1:19" ht="102.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="93" t="s">
         <v>123</v>
       </c>
-      <c r="B26" s="62"/>
-      <c r="C26" s="63" t="s">
+      <c r="B26" s="94"/>
+      <c r="C26" s="95" t="s">
         <v>197</v>
       </c>
-      <c r="D26" s="63"/>
-      <c r="E26" s="63"/>
-      <c r="F26" s="63"/>
-      <c r="G26" s="63"/>
+      <c r="D26" s="95"/>
+      <c r="E26" s="95"/>
+      <c r="F26" s="95"/>
+      <c r="G26" s="95"/>
       <c r="H26" s="36" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosAgenda</v>
@@ -5396,12 +5396,12 @@
       <c r="K26" s="49" t="s">
         <v>124</v>
       </c>
-      <c r="L26" s="64" t="s">
+      <c r="L26" s="96" t="s">
         <v>201</v>
       </c>
-      <c r="M26" s="64"/>
-      <c r="N26" s="64"/>
-      <c r="O26" s="64"/>
+      <c r="M26" s="96"/>
+      <c r="N26" s="96"/>
+      <c r="O26" s="96"/>
       <c r="P26" s="23" t="s">
         <v>192</v>
       </c>
@@ -5411,22 +5411,22 @@
       <c r="R26" s="37" t="s">
         <v>121</v>
       </c>
-      <c r="S26" s="111" t="s">
+      <c r="S26" s="54" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A27" s="65" t="s">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A27" s="97" t="s">
         <v>127</v>
       </c>
-      <c r="B27" s="66"/>
-      <c r="C27" s="67" t="s">
+      <c r="B27" s="98"/>
+      <c r="C27" s="99" t="s">
         <v>199</v>
       </c>
-      <c r="D27" s="67"/>
-      <c r="E27" s="67"/>
-      <c r="F27" s="67"/>
-      <c r="G27" s="67"/>
+      <c r="D27" s="99"/>
+      <c r="E27" s="99"/>
+      <c r="F27" s="99"/>
+      <c r="G27" s="99"/>
       <c r="H27" s="39" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosAgenda</v>
@@ -5440,39 +5440,39 @@
         <v>Corresponde a los datos que se van a modificar de la Agenda</v>
       </c>
       <c r="K27" s="41"/>
-      <c r="L27" s="112"/>
-      <c r="M27" s="113"/>
-      <c r="N27" s="113"/>
-      <c r="O27" s="114"/>
-      <c r="P27" s="115" t="s">
+      <c r="L27" s="100"/>
+      <c r="M27" s="101"/>
+      <c r="N27" s="101"/>
+      <c r="O27" s="102"/>
+      <c r="P27" s="72" t="s">
         <v>193</v>
       </c>
-      <c r="Q27" s="116" t="s">
+      <c r="Q27" s="74" t="s">
         <v>130</v>
       </c>
-      <c r="R27" s="116" t="s">
+      <c r="R27" s="74" t="s">
         <v>131</v>
       </c>
-      <c r="S27" s="117" t="s">
+      <c r="S27" s="76" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="90.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="58" t="s">
+    <row r="28" spans="1:19" ht="90.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="78" t="s">
         <v>133</v>
       </c>
-      <c r="B28" s="59"/>
-      <c r="C28" s="60" t="s">
+      <c r="B28" s="79"/>
+      <c r="C28" s="80" t="s">
         <v>200</v>
       </c>
-      <c r="D28" s="60"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="60"/>
-      <c r="G28" s="60"/>
-      <c r="H28" s="118" t="s">
+      <c r="D28" s="80"/>
+      <c r="E28" s="80"/>
+      <c r="F28" s="80"/>
+      <c r="G28" s="80"/>
+      <c r="H28" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="I28" s="119" t="s">
+      <c r="I28" s="56" t="s">
         <v>9</v>
       </c>
       <c r="J28" s="42" t="str">
@@ -5480,30 +5480,23 @@
         <v>Corresponde al identificador de la Agenda  que se quiere dar de baja.</v>
       </c>
       <c r="K28" s="43"/>
-      <c r="L28" s="120"/>
-      <c r="M28" s="121"/>
-      <c r="N28" s="121"/>
-      <c r="O28" s="122"/>
-      <c r="P28" s="123"/>
-      <c r="Q28" s="124"/>
-      <c r="R28" s="124"/>
-      <c r="S28" s="125"/>
+      <c r="L28" s="81"/>
+      <c r="M28" s="82"/>
+      <c r="N28" s="82"/>
+      <c r="O28" s="83"/>
+      <c r="P28" s="73"/>
+      <c r="Q28" s="75"/>
+      <c r="R28" s="75"/>
+      <c r="S28" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="R27:R28"/>
-    <mergeCell ref="S27:S28"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="L28:O28"/>
-    <mergeCell ref="P27:P28"/>
-    <mergeCell ref="Q27:Q28"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="L26:O26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="L27:O27"/>
+    <mergeCell ref="L21:O25"/>
+    <mergeCell ref="A21:B25"/>
+    <mergeCell ref="C21:G25"/>
+    <mergeCell ref="H21:H25"/>
+    <mergeCell ref="I21:I25"/>
+    <mergeCell ref="J21:J25"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="L20:O20"/>
     <mergeCell ref="A1:Q1"/>
@@ -5518,12 +5511,19 @@
     <mergeCell ref="K19:O19"/>
     <mergeCell ref="P19:Q19"/>
     <mergeCell ref="C14:C15"/>
-    <mergeCell ref="A21:B25"/>
-    <mergeCell ref="C21:G25"/>
-    <mergeCell ref="H21:H25"/>
-    <mergeCell ref="I21:I25"/>
-    <mergeCell ref="J21:J25"/>
-    <mergeCell ref="L21:O25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="L26:O26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="L27:O27"/>
+    <mergeCell ref="R27:R28"/>
+    <mergeCell ref="S27:S28"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="L28:O28"/>
+    <mergeCell ref="P27:P28"/>
+    <mergeCell ref="Q27:Q28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de Dominio'!A1" display="Volver al inicio" xr:uid="{B2E38F92-070F-4A08-9587-748CDC5E3622}"/>
@@ -5554,103 +5554,103 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC57795F-B02D-497B-A04E-44BC1D3D4128}">
   <dimension ref="A1:U27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" style="8" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" style="8" customWidth="1"/>
-    <col min="4" max="4" width="18.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="61.28515625" style="8" customWidth="1"/>
-    <col min="10" max="10" width="79.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" style="8" customWidth="1"/>
+    <col min="3" max="3" width="25.88671875" style="8" customWidth="1"/>
+    <col min="4" max="4" width="18.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="61.33203125" style="8" customWidth="1"/>
+    <col min="10" max="10" width="79.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.88671875" style="8" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="25" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="94.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="132.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="46.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="50.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="66.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="52.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="11.42578125" style="8"/>
+    <col min="17" max="17" width="94.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="132.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="46.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="50.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="66.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="52.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="11.44140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A1" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
-      <c r="H1" s="75"/>
-      <c r="I1" s="75"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
+      <c r="D1" s="121"/>
+      <c r="E1" s="121"/>
+      <c r="F1" s="121"/>
+      <c r="G1" s="121"/>
+      <c r="H1" s="121"/>
+      <c r="I1" s="121"/>
+      <c r="J1" s="121"/>
+      <c r="K1" s="121"/>
+      <c r="L1" s="121"/>
+      <c r="M1" s="121"/>
+      <c r="N1" s="121"/>
+      <c r="O1" s="121"/>
+      <c r="P1" s="121"/>
+      <c r="Q1" s="121"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="76" t="str">
+      <c r="B2" s="122" t="str">
         <f>'Listado Objetos de Dominio'!A5</f>
         <v>Turno</v>
       </c>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="76"/>
-      <c r="M2" s="76"/>
-      <c r="N2" s="76"/>
-      <c r="O2" s="76"/>
-      <c r="P2" s="76"/>
-      <c r="Q2" s="76"/>
-    </row>
-    <row r="3" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="122"/>
+      <c r="D2" s="122"/>
+      <c r="E2" s="122"/>
+      <c r="F2" s="122"/>
+      <c r="G2" s="122"/>
+      <c r="H2" s="122"/>
+      <c r="I2" s="122"/>
+      <c r="J2" s="122"/>
+      <c r="K2" s="122"/>
+      <c r="L2" s="122"/>
+      <c r="M2" s="122"/>
+      <c r="N2" s="122"/>
+      <c r="O2" s="122"/>
+      <c r="P2" s="122"/>
+      <c r="Q2" s="122"/>
+    </row>
+    <row r="3" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="77" t="str">
+      <c r="B3" s="123" t="str">
         <f>'Listado Objetos de Dominio'!B5</f>
         <v>Objeto de dominio que representa uno de los turnos que representan un bloque de tiempo que el residente podrá reservar.</v>
       </c>
-      <c r="C3" s="77"/>
-      <c r="D3" s="77"/>
-      <c r="E3" s="77"/>
-      <c r="F3" s="77"/>
-      <c r="G3" s="77"/>
-      <c r="H3" s="77"/>
-      <c r="I3" s="77"/>
-      <c r="J3" s="77"/>
-      <c r="K3" s="77"/>
-      <c r="L3" s="77"/>
-      <c r="M3" s="77"/>
-      <c r="N3" s="77"/>
-      <c r="O3" s="77"/>
-      <c r="P3" s="77"/>
-      <c r="Q3" s="77"/>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="C3" s="123"/>
+      <c r="D3" s="123"/>
+      <c r="E3" s="123"/>
+      <c r="F3" s="123"/>
+      <c r="G3" s="123"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
+      <c r="L3" s="123"/>
+      <c r="M3" s="123"/>
+      <c r="N3" s="123"/>
+      <c r="O3" s="123"/>
+      <c r="P3" s="123"/>
+      <c r="Q3" s="123"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>30</v>
       </c>
@@ -5702,24 +5702,24 @@
       <c r="Q4" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="R4" s="126" t="str">
+      <c r="R4" s="57" t="str">
         <f>A21</f>
         <v>Registrar</v>
       </c>
-      <c r="S4" s="127" t="str">
+      <c r="S4" s="58" t="str">
         <f>A25</f>
         <v>Buscar</v>
       </c>
-      <c r="T4" s="128" t="str">
+      <c r="T4" s="59" t="str">
         <f>A26</f>
         <v>Modificar</v>
       </c>
-      <c r="U4" s="129" t="str">
+      <c r="U4" s="60" t="str">
         <f>A27</f>
         <v>Eliminar</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
         <v>46</v>
       </c>
@@ -5759,7 +5759,7 @@
       <c r="Q5" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="R5" s="130" t="s">
+      <c r="R5" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S5" s="23" t="s">
@@ -5772,7 +5772,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A6" s="26" t="s">
         <v>109</v>
       </c>
@@ -5814,7 +5814,7 @@
       <c r="Q6" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="R6" s="130" t="s">
+      <c r="R6" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S6" s="23" t="s">
@@ -5827,7 +5827,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
         <v>83</v>
       </c>
@@ -5863,7 +5863,7 @@
       <c r="Q7" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="R7" s="130" t="s">
+      <c r="R7" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S7" s="23" t="s">
@@ -5876,7 +5876,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A8" s="26" t="s">
         <v>84</v>
       </c>
@@ -5912,7 +5912,7 @@
       <c r="Q8" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="R8" s="130" t="s">
+      <c r="R8" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S8" s="23" t="s">
@@ -5925,7 +5925,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>110</v>
       </c>
@@ -5961,7 +5961,7 @@
       <c r="Q9" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="R9" s="130" t="s">
+      <c r="R9" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S9" s="23" t="s">
@@ -5974,7 +5974,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="48" t="s">
         <v>85</v>
       </c>
@@ -6008,7 +6008,7 @@
       <c r="Q10" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="R10" s="130" t="s">
+      <c r="R10" s="61" t="s">
         <v>135</v>
       </c>
       <c r="S10" s="37" t="s">
@@ -6021,15 +6021,15 @@
         <v>140</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="72" t="s">
+    <row r="11" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:21" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="118" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="73"/>
-      <c r="C12" s="74"/>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B12" s="119"/>
+      <c r="C12" s="120"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" s="27" t="s">
         <v>53</v>
       </c>
@@ -6040,80 +6040,80 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="78" t="s">
+    <row r="14" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="130" t="s">
         <v>118</v>
       </c>
-      <c r="B14" s="80" t="s">
+      <c r="B14" s="126" t="s">
         <v>117</v>
       </c>
       <c r="C14" s="30" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="82"/>
-      <c r="B15" s="83"/>
+    <row r="15" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="131"/>
+      <c r="B15" s="133"/>
       <c r="C15" s="30" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="82"/>
-      <c r="B16" s="83"/>
+    <row r="16" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="131"/>
+      <c r="B16" s="133"/>
       <c r="C16" s="30" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="20.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="79"/>
-      <c r="B17" s="81"/>
+    <row r="17" spans="1:19" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="132"/>
+      <c r="B17" s="127"/>
       <c r="C17" s="46" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A19" s="68" t="s">
+    <row r="18" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A19" s="128" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="57"/>
-      <c r="C19" s="57" t="s">
+      <c r="B19" s="115"/>
+      <c r="C19" s="115" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="57"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="57"/>
-      <c r="G19" s="57"/>
-      <c r="H19" s="57" t="s">
+      <c r="D19" s="115"/>
+      <c r="E19" s="115"/>
+      <c r="F19" s="115"/>
+      <c r="G19" s="115"/>
+      <c r="H19" s="115" t="s">
         <v>56</v>
       </c>
-      <c r="I19" s="57"/>
-      <c r="J19" s="57"/>
-      <c r="K19" s="57" t="s">
+      <c r="I19" s="115"/>
+      <c r="J19" s="115"/>
+      <c r="K19" s="115" t="s">
         <v>57</v>
       </c>
-      <c r="L19" s="57"/>
-      <c r="M19" s="57"/>
-      <c r="N19" s="57"/>
-      <c r="O19" s="57"/>
-      <c r="P19" s="57" t="s">
+      <c r="L19" s="115"/>
+      <c r="M19" s="115"/>
+      <c r="N19" s="115"/>
+      <c r="O19" s="115"/>
+      <c r="P19" s="115" t="s">
         <v>58</v>
       </c>
-      <c r="Q19" s="57"/>
-      <c r="R19" s="57" t="s">
+      <c r="Q19" s="115"/>
+      <c r="R19" s="115" t="s">
         <v>59</v>
       </c>
-      <c r="S19" s="71"/>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A20" s="69"/>
-      <c r="B20" s="70"/>
-      <c r="C20" s="70"/>
-      <c r="D20" s="70"/>
-      <c r="E20" s="70"/>
-      <c r="F20" s="70"/>
-      <c r="G20" s="70"/>
+      <c r="S19" s="116"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A20" s="129"/>
+      <c r="B20" s="117"/>
+      <c r="C20" s="117"/>
+      <c r="D20" s="117"/>
+      <c r="E20" s="117"/>
+      <c r="F20" s="117"/>
+      <c r="G20" s="117"/>
       <c r="H20" s="32" t="s">
         <v>60</v>
       </c>
@@ -6126,12 +6126,12 @@
       <c r="K20" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="L20" s="70" t="s">
+      <c r="L20" s="117" t="s">
         <v>2</v>
       </c>
-      <c r="M20" s="70"/>
-      <c r="N20" s="70"/>
-      <c r="O20" s="70"/>
+      <c r="M20" s="117"/>
+      <c r="N20" s="117"/>
+      <c r="O20" s="117"/>
       <c r="P20" s="32" t="s">
         <v>62</v>
       </c>
@@ -6145,35 +6145,35 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="86" t="s">
+    <row r="21" spans="1:19" ht="151.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="103" t="s">
         <v>119</v>
       </c>
-      <c r="B21" s="87"/>
-      <c r="C21" s="88" t="s">
+      <c r="B21" s="104"/>
+      <c r="C21" s="84" t="s">
         <v>173</v>
       </c>
-      <c r="D21" s="89"/>
-      <c r="E21" s="89"/>
-      <c r="F21" s="89"/>
-      <c r="G21" s="90"/>
-      <c r="H21" s="54" t="str">
+      <c r="D21" s="85"/>
+      <c r="E21" s="85"/>
+      <c r="F21" s="85"/>
+      <c r="G21" s="86"/>
+      <c r="H21" s="69" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosTurno</v>
       </c>
-      <c r="I21" s="91" t="str">
+      <c r="I21" s="109" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosTurno</v>
       </c>
-      <c r="J21" s="92" t="str">
+      <c r="J21" s="112" t="str">
         <f>_xlfn.CONCAT("Corresponde al objeto que internamente contiene los datos necesarios para crear una nueva ",$B$2,)</f>
         <v>Corresponde al objeto que internamente contiene los datos necesarios para crear una nueva Turno</v>
       </c>
-      <c r="K21" s="93"/>
-      <c r="L21" s="88"/>
-      <c r="M21" s="89"/>
-      <c r="N21" s="89"/>
-      <c r="O21" s="90"/>
+      <c r="K21" s="50"/>
+      <c r="L21" s="84"/>
+      <c r="M21" s="85"/>
+      <c r="N21" s="85"/>
+      <c r="O21" s="86"/>
       <c r="P21" s="14" t="s">
         <v>165</v>
       </c>
@@ -6183,26 +6183,26 @@
       <c r="R21" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="S21" s="94" t="s">
+      <c r="S21" s="51" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="95"/>
-      <c r="B22" s="96"/>
-      <c r="C22" s="97"/>
-      <c r="D22" s="98"/>
-      <c r="E22" s="98"/>
-      <c r="F22" s="98"/>
-      <c r="G22" s="99"/>
-      <c r="H22" s="55"/>
-      <c r="I22" s="100"/>
-      <c r="J22" s="101"/>
-      <c r="K22" s="102"/>
-      <c r="L22" s="97"/>
-      <c r="M22" s="98"/>
-      <c r="N22" s="98"/>
-      <c r="O22" s="99"/>
+    <row r="22" spans="1:19" ht="151.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="105"/>
+      <c r="B22" s="106"/>
+      <c r="C22" s="87"/>
+      <c r="D22" s="88"/>
+      <c r="E22" s="88"/>
+      <c r="F22" s="88"/>
+      <c r="G22" s="89"/>
+      <c r="H22" s="70"/>
+      <c r="I22" s="110"/>
+      <c r="J22" s="113"/>
+      <c r="K22" s="52"/>
+      <c r="L22" s="87"/>
+      <c r="M22" s="88"/>
+      <c r="N22" s="88"/>
+      <c r="O22" s="89"/>
       <c r="P22" s="14" t="s">
         <v>166</v>
       </c>
@@ -6212,26 +6212,26 @@
       <c r="R22" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="S22" s="94" t="s">
+      <c r="S22" s="51" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="95"/>
-      <c r="B23" s="96"/>
-      <c r="C23" s="97"/>
-      <c r="D23" s="98"/>
-      <c r="E23" s="98"/>
-      <c r="F23" s="98"/>
-      <c r="G23" s="99"/>
-      <c r="H23" s="55"/>
-      <c r="I23" s="100"/>
-      <c r="J23" s="101"/>
-      <c r="K23" s="102"/>
-      <c r="L23" s="97"/>
-      <c r="M23" s="98"/>
-      <c r="N23" s="98"/>
-      <c r="O23" s="99"/>
+    <row r="23" spans="1:19" ht="75.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="105"/>
+      <c r="B23" s="106"/>
+      <c r="C23" s="87"/>
+      <c r="D23" s="88"/>
+      <c r="E23" s="88"/>
+      <c r="F23" s="88"/>
+      <c r="G23" s="89"/>
+      <c r="H23" s="70"/>
+      <c r="I23" s="110"/>
+      <c r="J23" s="113"/>
+      <c r="K23" s="52"/>
+      <c r="L23" s="87"/>
+      <c r="M23" s="88"/>
+      <c r="N23" s="88"/>
+      <c r="O23" s="89"/>
       <c r="P23" s="14" t="s">
         <v>167</v>
       </c>
@@ -6241,26 +6241,26 @@
       <c r="R23" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="S23" s="94" t="s">
+      <c r="S23" s="51" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="103"/>
-      <c r="B24" s="104"/>
-      <c r="C24" s="105"/>
-      <c r="D24" s="106"/>
-      <c r="E24" s="106"/>
-      <c r="F24" s="106"/>
-      <c r="G24" s="107"/>
-      <c r="H24" s="56"/>
-      <c r="I24" s="108"/>
-      <c r="J24" s="109"/>
-      <c r="K24" s="110"/>
-      <c r="L24" s="105"/>
-      <c r="M24" s="106"/>
-      <c r="N24" s="106"/>
-      <c r="O24" s="107"/>
+    <row r="24" spans="1:19" ht="77.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="107"/>
+      <c r="B24" s="108"/>
+      <c r="C24" s="90"/>
+      <c r="D24" s="91"/>
+      <c r="E24" s="91"/>
+      <c r="F24" s="91"/>
+      <c r="G24" s="92"/>
+      <c r="H24" s="71"/>
+      <c r="I24" s="111"/>
+      <c r="J24" s="114"/>
+      <c r="K24" s="53"/>
+      <c r="L24" s="90"/>
+      <c r="M24" s="91"/>
+      <c r="N24" s="91"/>
+      <c r="O24" s="92"/>
       <c r="P24" s="14" t="s">
         <v>168</v>
       </c>
@@ -6270,22 +6270,22 @@
       <c r="R24" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="S24" s="94" t="s">
+      <c r="S24" s="51" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="61" t="s">
+    <row r="25" spans="1:19" ht="105" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="93" t="s">
         <v>123</v>
       </c>
-      <c r="B25" s="62"/>
-      <c r="C25" s="63" t="s">
+      <c r="B25" s="94"/>
+      <c r="C25" s="95" t="s">
         <v>176</v>
       </c>
-      <c r="D25" s="63"/>
-      <c r="E25" s="63"/>
-      <c r="F25" s="63"/>
-      <c r="G25" s="63"/>
+      <c r="D25" s="95"/>
+      <c r="E25" s="95"/>
+      <c r="F25" s="95"/>
+      <c r="G25" s="95"/>
       <c r="H25" s="36" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosTurno</v>
@@ -6301,12 +6301,12 @@
       <c r="K25" s="49" t="s">
         <v>124</v>
       </c>
-      <c r="L25" s="64" t="s">
+      <c r="L25" s="96" t="s">
         <v>182</v>
       </c>
-      <c r="M25" s="64"/>
-      <c r="N25" s="64"/>
-      <c r="O25" s="64"/>
+      <c r="M25" s="96"/>
+      <c r="N25" s="96"/>
+      <c r="O25" s="96"/>
       <c r="P25" s="23" t="s">
         <v>183</v>
       </c>
@@ -6316,22 +6316,22 @@
       <c r="R25" s="37" t="s">
         <v>121</v>
       </c>
-      <c r="S25" s="111" t="s">
+      <c r="S25" s="54" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="65" t="s">
+    <row r="26" spans="1:19" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="97" t="s">
         <v>127</v>
       </c>
-      <c r="B26" s="66"/>
-      <c r="C26" s="67" t="s">
+      <c r="B26" s="98"/>
+      <c r="C26" s="99" t="s">
         <v>174</v>
       </c>
-      <c r="D26" s="67"/>
-      <c r="E26" s="67"/>
-      <c r="F26" s="67"/>
-      <c r="G26" s="67"/>
+      <c r="D26" s="99"/>
+      <c r="E26" s="99"/>
+      <c r="F26" s="99"/>
+      <c r="G26" s="99"/>
       <c r="H26" s="39" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosTurno</v>
@@ -6345,39 +6345,39 @@
         <v>Corresponde a los datos que se van a modificar de la Turno</v>
       </c>
       <c r="K26" s="41"/>
-      <c r="L26" s="112"/>
-      <c r="M26" s="113"/>
-      <c r="N26" s="113"/>
-      <c r="O26" s="114"/>
-      <c r="P26" s="133" t="s">
+      <c r="L26" s="100"/>
+      <c r="M26" s="101"/>
+      <c r="N26" s="101"/>
+      <c r="O26" s="102"/>
+      <c r="P26" s="62" t="s">
         <v>184</v>
       </c>
-      <c r="Q26" s="134" t="s">
+      <c r="Q26" s="63" t="s">
         <v>130</v>
       </c>
-      <c r="R26" s="134" t="s">
+      <c r="R26" s="63" t="s">
         <v>131</v>
       </c>
-      <c r="S26" s="135" t="s">
+      <c r="S26" s="64" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="58" t="s">
+    <row r="27" spans="1:19" ht="84.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="78" t="s">
         <v>133</v>
       </c>
-      <c r="B27" s="59"/>
-      <c r="C27" s="60" t="s">
+      <c r="B27" s="79"/>
+      <c r="C27" s="80" t="s">
         <v>175</v>
       </c>
-      <c r="D27" s="60"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="60"/>
-      <c r="G27" s="60"/>
-      <c r="H27" s="118" t="s">
+      <c r="D27" s="80"/>
+      <c r="E27" s="80"/>
+      <c r="F27" s="80"/>
+      <c r="G27" s="80"/>
+      <c r="H27" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="I27" s="119" t="s">
+      <c r="I27" s="56" t="s">
         <v>9</v>
       </c>
       <c r="J27" s="42" t="str">
@@ -6385,10 +6385,10 @@
         <v>Corresponde al identificador de la Turno  que se quiere dar de baja.</v>
       </c>
       <c r="K27" s="43"/>
-      <c r="L27" s="120"/>
-      <c r="M27" s="121"/>
-      <c r="N27" s="121"/>
-      <c r="O27" s="122"/>
+      <c r="L27" s="81"/>
+      <c r="M27" s="82"/>
+      <c r="N27" s="82"/>
+      <c r="O27" s="83"/>
       <c r="P27" s="44" t="s">
         <v>184</v>
       </c>
@@ -6404,15 +6404,12 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="L27:O27"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="L25:O25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="L26:O26"/>
+    <mergeCell ref="L21:O24"/>
+    <mergeCell ref="A21:B24"/>
+    <mergeCell ref="C21:G24"/>
+    <mergeCell ref="H21:H24"/>
+    <mergeCell ref="I21:I24"/>
+    <mergeCell ref="J21:J24"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="L20:O20"/>
     <mergeCell ref="A1:Q1"/>
@@ -6426,12 +6423,15 @@
     <mergeCell ref="H19:J19"/>
     <mergeCell ref="K19:O19"/>
     <mergeCell ref="P19:Q19"/>
-    <mergeCell ref="A21:B24"/>
-    <mergeCell ref="C21:G24"/>
-    <mergeCell ref="H21:H24"/>
-    <mergeCell ref="I21:I24"/>
-    <mergeCell ref="J21:J24"/>
-    <mergeCell ref="L21:O24"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="L27:O27"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="L25:O25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="L26:O26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de Dominio'!A1" display="Volver al inicio" xr:uid="{186E73A2-C89F-4A82-8727-EBDE505719F2}"/>

</xml_diff>

<commit_message>
Modifique las relaciones entre contextos Residente ConjuntosResidenciales 0001 , Agenda ConjuntoResidenciales0001 , Reserva-0001 y Reserva-0002y se crearon lo nuevos enriquesidos para tipoInmueble, TipoZonaInmueble y UnidadTiempoUso
</commit_message>
<xml_diff>
--- a/Doo-Doc/Nueva Version Victus/Modelos de Dominio Enriquecidos/Modelo De Dominio Enriquecido Agendas.xlsx
+++ b/Doo-Doc/Nueva Version Victus/Modelos de Dominio Enriquecidos/Modelo De Dominio Enriquecido Agendas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\DOO 2024 BD\DOO\victus-doc\Doo-Doc\Nueva Version Victus\Modelos de Dominio Enriquecidos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA236762-3ED3-439A-B8E7-742C55D62F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C174E49-CBBB-432D-8801-C25A97A621A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="4" xr2:uid="{9E75F319-B909-453D-9AFC-FA9C5B40B20E}"/>
+    <workbookView xWindow="19395" yWindow="1995" windowWidth="19095" windowHeight="15345" firstSheet="2" activeTab="5" xr2:uid="{9E75F319-B909-453D-9AFC-FA9C5B40B20E}"/>
   </bookViews>
   <sheets>
     <sheet name="Valores" sheetId="1" r:id="rId1"/>
@@ -1331,7 +1331,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="209">
   <si>
     <t>Tipo Objeto Dominio</t>
   </si>
@@ -2799,6 +2799,144 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2834,144 +2972,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="28" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3087,8 +3087,11 @@
       <sheetName val="Listado Objetos Dominio"/>
       <sheetName val="ConjuntoResidencial"/>
       <sheetName val="ZonaComun"/>
+      <sheetName val="UnidadTiempoUso"/>
       <sheetName val="Administrador"/>
       <sheetName val="ZonaInmueble"/>
+      <sheetName val="TipoZonaInmueble"/>
+      <sheetName val="TipoInmueble"/>
       <sheetName val="Inmueble"/>
     </sheetNames>
     <sheetDataSet>
@@ -3109,6 +3112,9 @@
       <sheetData sheetId="5" refreshError="1"/>
       <sheetData sheetId="6" refreshError="1"/>
       <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -3432,19 +3438,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AC31824-1358-4896-8FEC-CA18F2D1F29C}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="65" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="66"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -3452,7 +3458,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
@@ -3460,7 +3466,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
@@ -3468,52 +3474,52 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>15</v>
       </c>
@@ -3529,7 +3535,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{270AC7B1-5317-4DF0-8E73-05A502D22732}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3539,16 +3545,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6DC33F5-6024-4ECE-8864-A6190D431B22}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="56.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="11.44140625" style="8"/>
+    <col min="1" max="1" width="21.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="56.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="11.42578125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>16</v>
       </c>
@@ -3558,7 +3564,7 @@
       <c r="C1" s="67"/>
       <c r="D1" s="68"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>17</v>
       </c>
@@ -3572,7 +3578,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>20</v>
       </c>
@@ -3587,7 +3593,7 @@
         <v>Agendas</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
         <v>21</v>
       </c>
@@ -3599,7 +3605,7 @@
       </c>
       <c r="D4" s="70"/>
     </row>
-    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>22</v>
       </c>
@@ -3628,103 +3634,103 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0BC2B36-176F-457B-9E5A-2C1354FBA2A7}">
   <dimension ref="A1:U27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5546875" style="8" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="61.33203125" style="8" customWidth="1"/>
-    <col min="10" max="10" width="79.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="61.28515625" style="8" customWidth="1"/>
+    <col min="10" max="10" width="79.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.85546875" style="8" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="25" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="94.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="39.6640625" style="8" customWidth="1"/>
-    <col min="19" max="19" width="46.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="32.44140625" style="8" customWidth="1"/>
-    <col min="21" max="21" width="25.44140625" style="8" customWidth="1"/>
-    <col min="22" max="22" width="52.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="11.44140625" style="8"/>
+    <col min="17" max="17" width="94.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="39.7109375" style="8" customWidth="1"/>
+    <col min="19" max="19" width="46.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="32.42578125" style="8" customWidth="1"/>
+    <col min="21" max="21" width="25.42578125" style="8" customWidth="1"/>
+    <col min="22" max="22" width="52.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="11.42578125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A1" s="121" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A1" s="78" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
-      <c r="F1" s="121"/>
-      <c r="G1" s="121"/>
-      <c r="H1" s="121"/>
-      <c r="I1" s="121"/>
-      <c r="J1" s="121"/>
-      <c r="K1" s="121"/>
-      <c r="L1" s="121"/>
-      <c r="M1" s="121"/>
-      <c r="N1" s="121"/>
-      <c r="O1" s="121"/>
-      <c r="P1" s="121"/>
-      <c r="Q1" s="121"/>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
+      <c r="P1" s="78"/>
+      <c r="Q1" s="78"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="122" t="str">
+      <c r="B2" s="79" t="str">
         <f>'[1]Listado Objetos Dominio'!A4</f>
         <v>ZonaComun</v>
       </c>
-      <c r="C2" s="122"/>
-      <c r="D2" s="122"/>
-      <c r="E2" s="122"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="122"/>
-      <c r="H2" s="122"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="122"/>
-      <c r="K2" s="122"/>
-      <c r="L2" s="122"/>
-      <c r="M2" s="122"/>
-      <c r="N2" s="122"/>
-      <c r="O2" s="122"/>
-      <c r="P2" s="122"/>
-      <c r="Q2" s="122"/>
-    </row>
-    <row r="3" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="79"/>
+      <c r="M2" s="79"/>
+      <c r="N2" s="79"/>
+      <c r="O2" s="79"/>
+      <c r="P2" s="79"/>
+      <c r="Q2" s="79"/>
+    </row>
+    <row r="3" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="123" t="str">
+      <c r="B3" s="80" t="str">
         <f>'[1]Listado Objetos Dominio'!B4</f>
         <v>Objeto de dominio que representa a cada una de las zonas comunes que se encuentran dentro de un conjunto residencial para que los residentes puedan reservar esos espacios y poder usarlos.</v>
       </c>
-      <c r="C3" s="123"/>
-      <c r="D3" s="123"/>
-      <c r="E3" s="123"/>
-      <c r="F3" s="123"/>
-      <c r="G3" s="123"/>
-      <c r="H3" s="123"/>
-      <c r="I3" s="123"/>
-      <c r="J3" s="123"/>
-      <c r="K3" s="123"/>
-      <c r="L3" s="123"/>
-      <c r="M3" s="123"/>
-      <c r="N3" s="123"/>
-      <c r="O3" s="123"/>
-      <c r="P3" s="123"/>
-      <c r="Q3" s="123"/>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="80"/>
+      <c r="L3" s="80"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="80"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="80"/>
+      <c r="Q3" s="80"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>30</v>
       </c>
@@ -3793,7 +3799,7 @@
         <v>Eliminar</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
         <v>46</v>
       </c>
@@ -3846,7 +3852,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
         <v>50</v>
       </c>
@@ -3901,7 +3907,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
         <v>66</v>
       </c>
@@ -3956,7 +3962,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
         <v>87</v>
       </c>
@@ -4005,7 +4011,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
         <v>88</v>
       </c>
@@ -4056,7 +4062,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="26" t="s">
         <v>89</v>
       </c>
@@ -4105,7 +4111,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
         <v>67</v>
       </c>
@@ -4160,7 +4166,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="45" t="s">
         <v>68</v>
       </c>
@@ -4207,15 +4213,15 @@
         <v>140</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="14" spans="1:21" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="118" t="s">
+    <row r="13" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="75" t="s">
         <v>98</v>
       </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="120"/>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B14" s="76"/>
+      <c r="C14" s="77"/>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
         <v>53</v>
       </c>
@@ -4226,66 +4232,66 @@
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="124" t="s">
+    <row r="16" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="81" t="s">
         <v>99</v>
       </c>
-      <c r="B16" s="126" t="s">
+      <c r="B16" s="83" t="s">
         <v>100</v>
       </c>
       <c r="C16" s="30" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="125"/>
-      <c r="B17" s="127"/>
+    <row r="17" spans="1:19" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="82"/>
+      <c r="B17" s="84"/>
       <c r="C17" s="31" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A19" s="128" t="s">
+    <row r="18" spans="1:19" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A19" s="85" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="115"/>
-      <c r="C19" s="115" t="s">
+      <c r="B19" s="72"/>
+      <c r="C19" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="115"/>
-      <c r="E19" s="115"/>
-      <c r="F19" s="115"/>
-      <c r="G19" s="115"/>
-      <c r="H19" s="115" t="s">
+      <c r="D19" s="72"/>
+      <c r="E19" s="72"/>
+      <c r="F19" s="72"/>
+      <c r="G19" s="72"/>
+      <c r="H19" s="72" t="s">
         <v>56</v>
       </c>
-      <c r="I19" s="115"/>
-      <c r="J19" s="115"/>
-      <c r="K19" s="115" t="s">
+      <c r="I19" s="72"/>
+      <c r="J19" s="72"/>
+      <c r="K19" s="72" t="s">
         <v>57</v>
       </c>
-      <c r="L19" s="115"/>
-      <c r="M19" s="115"/>
-      <c r="N19" s="115"/>
-      <c r="O19" s="115"/>
-      <c r="P19" s="115" t="s">
+      <c r="L19" s="72"/>
+      <c r="M19" s="72"/>
+      <c r="N19" s="72"/>
+      <c r="O19" s="72"/>
+      <c r="P19" s="72" t="s">
         <v>58</v>
       </c>
-      <c r="Q19" s="115"/>
-      <c r="R19" s="115" t="s">
+      <c r="Q19" s="72"/>
+      <c r="R19" s="72" t="s">
         <v>59</v>
       </c>
-      <c r="S19" s="116"/>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A20" s="129"/>
-      <c r="B20" s="117"/>
-      <c r="C20" s="117"/>
-      <c r="D20" s="117"/>
-      <c r="E20" s="117"/>
-      <c r="F20" s="117"/>
-      <c r="G20" s="117"/>
+      <c r="S19" s="73"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20" s="86"/>
+      <c r="B20" s="74"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="74"/>
+      <c r="E20" s="74"/>
+      <c r="F20" s="74"/>
+      <c r="G20" s="74"/>
       <c r="H20" s="32" t="s">
         <v>60</v>
       </c>
@@ -4298,12 +4304,12 @@
       <c r="K20" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="L20" s="117" t="s">
+      <c r="L20" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="M20" s="117"/>
-      <c r="N20" s="117"/>
-      <c r="O20" s="117"/>
+      <c r="M20" s="74"/>
+      <c r="N20" s="74"/>
+      <c r="O20" s="74"/>
       <c r="P20" s="32" t="s">
         <v>62</v>
       </c>
@@ -4317,32 +4323,32 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="103" t="s">
+    <row r="21" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+      <c r="A21" s="106" t="s">
         <v>119</v>
       </c>
-      <c r="B21" s="104"/>
-      <c r="C21" s="84" t="s">
+      <c r="B21" s="107"/>
+      <c r="C21" s="87" t="s">
         <v>120</v>
       </c>
-      <c r="D21" s="85"/>
-      <c r="E21" s="85"/>
-      <c r="F21" s="85"/>
-      <c r="G21" s="86"/>
+      <c r="D21" s="88"/>
+      <c r="E21" s="88"/>
+      <c r="F21" s="88"/>
+      <c r="G21" s="89"/>
       <c r="H21" s="69" t="s">
         <v>144</v>
       </c>
-      <c r="I21" s="109" t="s">
+      <c r="I21" s="112" t="s">
         <v>20</v>
       </c>
-      <c r="J21" s="112" t="s">
+      <c r="J21" s="115" t="s">
         <v>145</v>
       </c>
       <c r="K21" s="50"/>
-      <c r="L21" s="84"/>
-      <c r="M21" s="85"/>
-      <c r="N21" s="85"/>
-      <c r="O21" s="86"/>
+      <c r="L21" s="87"/>
+      <c r="M21" s="88"/>
+      <c r="N21" s="88"/>
+      <c r="O21" s="89"/>
       <c r="P21" s="14" t="s">
         <v>146</v>
       </c>
@@ -4356,22 +4362,22 @@
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="105"/>
-      <c r="B22" s="106"/>
-      <c r="C22" s="87"/>
-      <c r="D22" s="88"/>
-      <c r="E22" s="88"/>
-      <c r="F22" s="88"/>
-      <c r="G22" s="89"/>
+    <row r="22" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+      <c r="A22" s="108"/>
+      <c r="B22" s="109"/>
+      <c r="C22" s="90"/>
+      <c r="D22" s="91"/>
+      <c r="E22" s="91"/>
+      <c r="F22" s="91"/>
+      <c r="G22" s="92"/>
       <c r="H22" s="70"/>
-      <c r="I22" s="110"/>
-      <c r="J22" s="113"/>
+      <c r="I22" s="113"/>
+      <c r="J22" s="116"/>
       <c r="K22" s="52"/>
-      <c r="L22" s="87"/>
-      <c r="M22" s="88"/>
-      <c r="N22" s="88"/>
-      <c r="O22" s="89"/>
+      <c r="L22" s="90"/>
+      <c r="M22" s="91"/>
+      <c r="N22" s="91"/>
+      <c r="O22" s="92"/>
       <c r="P22" s="14" t="s">
         <v>148</v>
       </c>
@@ -4385,22 +4391,22 @@
         <v>151</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="105"/>
-      <c r="B23" s="106"/>
-      <c r="C23" s="87"/>
-      <c r="D23" s="88"/>
-      <c r="E23" s="88"/>
-      <c r="F23" s="88"/>
-      <c r="G23" s="89"/>
+    <row r="23" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" s="108"/>
+      <c r="B23" s="109"/>
+      <c r="C23" s="90"/>
+      <c r="D23" s="91"/>
+      <c r="E23" s="91"/>
+      <c r="F23" s="91"/>
+      <c r="G23" s="92"/>
       <c r="H23" s="70"/>
-      <c r="I23" s="110"/>
-      <c r="J23" s="113"/>
+      <c r="I23" s="113"/>
+      <c r="J23" s="116"/>
       <c r="K23" s="52"/>
-      <c r="L23" s="87"/>
-      <c r="M23" s="88"/>
-      <c r="N23" s="88"/>
-      <c r="O23" s="89"/>
+      <c r="L23" s="90"/>
+      <c r="M23" s="91"/>
+      <c r="N23" s="91"/>
+      <c r="O23" s="92"/>
       <c r="P23" s="14" t="s">
         <v>152</v>
       </c>
@@ -4414,22 +4420,22 @@
         <v>155</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="72" x14ac:dyDescent="0.3">
-      <c r="A24" s="107"/>
-      <c r="B24" s="108"/>
-      <c r="C24" s="90"/>
-      <c r="D24" s="91"/>
-      <c r="E24" s="91"/>
-      <c r="F24" s="91"/>
-      <c r="G24" s="92"/>
+    <row r="24" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+      <c r="A24" s="110"/>
+      <c r="B24" s="111"/>
+      <c r="C24" s="93"/>
+      <c r="D24" s="94"/>
+      <c r="E24" s="94"/>
+      <c r="F24" s="94"/>
+      <c r="G24" s="95"/>
       <c r="H24" s="71"/>
-      <c r="I24" s="111"/>
-      <c r="J24" s="114"/>
+      <c r="I24" s="114"/>
+      <c r="J24" s="117"/>
       <c r="K24" s="53"/>
-      <c r="L24" s="90"/>
-      <c r="M24" s="91"/>
-      <c r="N24" s="91"/>
-      <c r="O24" s="92"/>
+      <c r="L24" s="93"/>
+      <c r="M24" s="94"/>
+      <c r="N24" s="94"/>
+      <c r="O24" s="95"/>
       <c r="P24" s="14" t="s">
         <v>156</v>
       </c>
@@ -4443,18 +4449,18 @@
         <v>159</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="93" t="s">
+    <row r="25" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+      <c r="A25" s="96" t="s">
         <v>123</v>
       </c>
-      <c r="B25" s="94"/>
-      <c r="C25" s="95" t="s">
+      <c r="B25" s="97"/>
+      <c r="C25" s="98" t="s">
         <v>160</v>
       </c>
-      <c r="D25" s="95"/>
-      <c r="E25" s="95"/>
-      <c r="F25" s="95"/>
-      <c r="G25" s="95"/>
+      <c r="D25" s="98"/>
+      <c r="E25" s="98"/>
+      <c r="F25" s="98"/>
+      <c r="G25" s="98"/>
       <c r="H25" s="36" t="s">
         <v>144</v>
       </c>
@@ -4467,12 +4473,12 @@
       <c r="K25" s="49" t="s">
         <v>124</v>
       </c>
-      <c r="L25" s="96" t="s">
+      <c r="L25" s="99" t="s">
         <v>125</v>
       </c>
-      <c r="M25" s="96"/>
-      <c r="N25" s="96"/>
-      <c r="O25" s="96"/>
+      <c r="M25" s="99"/>
+      <c r="N25" s="99"/>
+      <c r="O25" s="99"/>
       <c r="P25" s="23" t="s">
         <v>162</v>
       </c>
@@ -4486,18 +4492,18 @@
         <v>122</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A26" s="97" t="s">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A26" s="100" t="s">
         <v>127</v>
       </c>
-      <c r="B26" s="98"/>
-      <c r="C26" s="99" t="s">
+      <c r="B26" s="101"/>
+      <c r="C26" s="102" t="s">
         <v>128</v>
       </c>
-      <c r="D26" s="99"/>
-      <c r="E26" s="99"/>
-      <c r="F26" s="99"/>
-      <c r="G26" s="99"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="102"/>
+      <c r="F26" s="102"/>
+      <c r="G26" s="102"/>
       <c r="H26" s="39" t="s">
         <v>144</v>
       </c>
@@ -4508,35 +4514,35 @@
         <v>163</v>
       </c>
       <c r="K26" s="41"/>
-      <c r="L26" s="100"/>
-      <c r="M26" s="101"/>
-      <c r="N26" s="101"/>
-      <c r="O26" s="102"/>
-      <c r="P26" s="72" t="s">
+      <c r="L26" s="103"/>
+      <c r="M26" s="104"/>
+      <c r="N26" s="104"/>
+      <c r="O26" s="105"/>
+      <c r="P26" s="118" t="s">
         <v>129</v>
       </c>
-      <c r="Q26" s="74" t="s">
+      <c r="Q26" s="120" t="s">
         <v>130</v>
       </c>
-      <c r="R26" s="74" t="s">
+      <c r="R26" s="120" t="s">
         <v>131</v>
       </c>
-      <c r="S26" s="76" t="s">
+      <c r="S26" s="122" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A27" s="78" t="s">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A27" s="124" t="s">
         <v>133</v>
       </c>
-      <c r="B27" s="79"/>
-      <c r="C27" s="80" t="s">
+      <c r="B27" s="125"/>
+      <c r="C27" s="126" t="s">
         <v>134</v>
       </c>
-      <c r="D27" s="80"/>
-      <c r="E27" s="80"/>
-      <c r="F27" s="80"/>
-      <c r="G27" s="80"/>
+      <c r="D27" s="126"/>
+      <c r="E27" s="126"/>
+      <c r="F27" s="126"/>
+      <c r="G27" s="126"/>
       <c r="H27" s="55" t="s">
         <v>46</v>
       </c>
@@ -4547,17 +4553,36 @@
         <v>164</v>
       </c>
       <c r="K27" s="43"/>
-      <c r="L27" s="81"/>
-      <c r="M27" s="82"/>
-      <c r="N27" s="82"/>
-      <c r="O27" s="83"/>
-      <c r="P27" s="73"/>
-      <c r="Q27" s="75"/>
-      <c r="R27" s="75"/>
-      <c r="S27" s="77"/>
+      <c r="L27" s="127"/>
+      <c r="M27" s="128"/>
+      <c r="N27" s="128"/>
+      <c r="O27" s="129"/>
+      <c r="P27" s="119"/>
+      <c r="Q27" s="121"/>
+      <c r="R27" s="121"/>
+      <c r="S27" s="123"/>
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="P26:P27"/>
+    <mergeCell ref="Q26:Q27"/>
+    <mergeCell ref="R26:R27"/>
+    <mergeCell ref="S26:S27"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="L27:O27"/>
+    <mergeCell ref="L21:O24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="L25:O25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="L26:O26"/>
+    <mergeCell ref="A21:B24"/>
+    <mergeCell ref="C21:G24"/>
+    <mergeCell ref="H21:H24"/>
+    <mergeCell ref="I21:I24"/>
+    <mergeCell ref="J21:J24"/>
     <mergeCell ref="P19:Q19"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="L20:O20"/>
@@ -4571,25 +4596,6 @@
     <mergeCell ref="A19:B20"/>
     <mergeCell ref="C19:G20"/>
     <mergeCell ref="H19:J19"/>
-    <mergeCell ref="L21:O24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="L25:O25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="L26:O26"/>
-    <mergeCell ref="A21:B24"/>
-    <mergeCell ref="C21:G24"/>
-    <mergeCell ref="H21:H24"/>
-    <mergeCell ref="I21:I24"/>
-    <mergeCell ref="J21:J24"/>
-    <mergeCell ref="P26:P27"/>
-    <mergeCell ref="Q26:Q27"/>
-    <mergeCell ref="R26:R27"/>
-    <mergeCell ref="S26:S27"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="L27:O27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de Dominio'!A1" display="Volver al inicio" xr:uid="{86A492AF-8702-4148-85C2-41FF6CA10413}"/>
@@ -4618,103 +4624,103 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{037CC029-DC44-4605-90F4-CA51C57B9385}">
   <dimension ref="A1:U28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5546875" style="8" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="61.33203125" style="8" customWidth="1"/>
-    <col min="10" max="10" width="79.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="61.28515625" style="8" customWidth="1"/>
+    <col min="10" max="10" width="79.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.85546875" style="8" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="25" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="94.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="43.5546875" style="8" customWidth="1"/>
-    <col min="19" max="19" width="46.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="50.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="66.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="52.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="11.44140625" style="8"/>
+    <col min="17" max="17" width="94.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="43.5703125" style="8" customWidth="1"/>
+    <col min="19" max="19" width="46.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="50.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="66.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="52.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="11.42578125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A1" s="121" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A1" s="78" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
-      <c r="F1" s="121"/>
-      <c r="G1" s="121"/>
-      <c r="H1" s="121"/>
-      <c r="I1" s="121"/>
-      <c r="J1" s="121"/>
-      <c r="K1" s="121"/>
-      <c r="L1" s="121"/>
-      <c r="M1" s="121"/>
-      <c r="N1" s="121"/>
-      <c r="O1" s="121"/>
-      <c r="P1" s="121"/>
-      <c r="Q1" s="121"/>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
+      <c r="P1" s="78"/>
+      <c r="Q1" s="78"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="122" t="str">
+      <c r="B2" s="79" t="str">
         <f>'Listado Objetos de Dominio'!A4</f>
         <v>Agenda</v>
       </c>
-      <c r="C2" s="122"/>
-      <c r="D2" s="122"/>
-      <c r="E2" s="122"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="122"/>
-      <c r="H2" s="122"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="122"/>
-      <c r="K2" s="122"/>
-      <c r="L2" s="122"/>
-      <c r="M2" s="122"/>
-      <c r="N2" s="122"/>
-      <c r="O2" s="122"/>
-      <c r="P2" s="122"/>
-      <c r="Q2" s="122"/>
-    </row>
-    <row r="3" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="79"/>
+      <c r="M2" s="79"/>
+      <c r="N2" s="79"/>
+      <c r="O2" s="79"/>
+      <c r="P2" s="79"/>
+      <c r="Q2" s="79"/>
+    </row>
+    <row r="3" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="123" t="str">
+      <c r="B3" s="80" t="str">
         <f>'Listado Objetos de Dominio'!B4</f>
         <v>Objeto de dominio que representaa cada una de las agendas que dónde el residente podrá reservar.</v>
       </c>
-      <c r="C3" s="123"/>
-      <c r="D3" s="123"/>
-      <c r="E3" s="123"/>
-      <c r="F3" s="123"/>
-      <c r="G3" s="123"/>
-      <c r="H3" s="123"/>
-      <c r="I3" s="123"/>
-      <c r="J3" s="123"/>
-      <c r="K3" s="123"/>
-      <c r="L3" s="123"/>
-      <c r="M3" s="123"/>
-      <c r="N3" s="123"/>
-      <c r="O3" s="123"/>
-      <c r="P3" s="123"/>
-      <c r="Q3" s="123"/>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="80"/>
+      <c r="L3" s="80"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="80"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="80"/>
+      <c r="Q3" s="80"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>30</v>
       </c>
@@ -4783,7 +4789,7 @@
         <v>Eliminar</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
         <v>46</v>
       </c>
@@ -4836,7 +4842,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
         <v>50</v>
       </c>
@@ -4891,7 +4897,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
         <v>101</v>
       </c>
@@ -4942,7 +4948,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
         <v>69</v>
       </c>
@@ -4991,7 +4997,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
         <v>70</v>
       </c>
@@ -5040,7 +5046,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="47" t="s">
         <v>71</v>
       </c>
@@ -5055,9 +5061,7 @@
       <c r="H10" s="19"/>
       <c r="I10" s="20"/>
       <c r="J10" s="19"/>
-      <c r="K10" s="21" t="s">
-        <v>65</v>
-      </c>
+      <c r="K10" s="21"/>
       <c r="L10" s="22" t="s">
         <v>49</v>
       </c>
@@ -5089,15 +5093,15 @@
         <v>140</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="12" spans="1:21" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="118" t="s">
+    <row r="11" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="75" t="s">
         <v>98</v>
       </c>
-      <c r="B12" s="119"/>
-      <c r="C12" s="120"/>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B12" s="76"/>
+      <c r="C12" s="77"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
         <v>53</v>
       </c>
@@ -5108,78 +5112,78 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="130" t="s">
         <v>82</v>
       </c>
-      <c r="B14" s="126" t="s">
+      <c r="B14" s="83" t="s">
         <v>108</v>
       </c>
       <c r="C14" s="134" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="131"/>
       <c r="B15" s="133"/>
       <c r="C15" s="135"/>
     </row>
-    <row r="16" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="131"/>
       <c r="B16" s="133"/>
       <c r="C16" s="30" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:19" ht="20.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="132"/>
-      <c r="B17" s="127"/>
+      <c r="B17" s="84"/>
       <c r="C17" s="46" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A19" s="128" t="s">
+    <row r="18" spans="1:19" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A19" s="85" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="115"/>
-      <c r="C19" s="115" t="s">
+      <c r="B19" s="72"/>
+      <c r="C19" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="115"/>
-      <c r="E19" s="115"/>
-      <c r="F19" s="115"/>
-      <c r="G19" s="115"/>
-      <c r="H19" s="115" t="s">
+      <c r="D19" s="72"/>
+      <c r="E19" s="72"/>
+      <c r="F19" s="72"/>
+      <c r="G19" s="72"/>
+      <c r="H19" s="72" t="s">
         <v>56</v>
       </c>
-      <c r="I19" s="115"/>
-      <c r="J19" s="115"/>
-      <c r="K19" s="115" t="s">
+      <c r="I19" s="72"/>
+      <c r="J19" s="72"/>
+      <c r="K19" s="72" t="s">
         <v>57</v>
       </c>
-      <c r="L19" s="115"/>
-      <c r="M19" s="115"/>
-      <c r="N19" s="115"/>
-      <c r="O19" s="115"/>
-      <c r="P19" s="115" t="s">
+      <c r="L19" s="72"/>
+      <c r="M19" s="72"/>
+      <c r="N19" s="72"/>
+      <c r="O19" s="72"/>
+      <c r="P19" s="72" t="s">
         <v>58</v>
       </c>
-      <c r="Q19" s="115"/>
-      <c r="R19" s="115" t="s">
+      <c r="Q19" s="72"/>
+      <c r="R19" s="72" t="s">
         <v>59</v>
       </c>
-      <c r="S19" s="116"/>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A20" s="129"/>
-      <c r="B20" s="117"/>
-      <c r="C20" s="117"/>
-      <c r="D20" s="117"/>
-      <c r="E20" s="117"/>
-      <c r="F20" s="117"/>
-      <c r="G20" s="117"/>
+      <c r="S19" s="73"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20" s="86"/>
+      <c r="B20" s="74"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="74"/>
+      <c r="E20" s="74"/>
+      <c r="F20" s="74"/>
+      <c r="G20" s="74"/>
       <c r="H20" s="32" t="s">
         <v>60</v>
       </c>
@@ -5192,12 +5196,12 @@
       <c r="K20" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="L20" s="117" t="s">
+      <c r="L20" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="M20" s="117"/>
-      <c r="N20" s="117"/>
-      <c r="O20" s="117"/>
+      <c r="M20" s="74"/>
+      <c r="N20" s="74"/>
+      <c r="O20" s="74"/>
       <c r="P20" s="32" t="s">
         <v>62</v>
       </c>
@@ -5211,35 +5215,35 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="87" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="103" t="s">
+    <row r="21" spans="1:19" ht="87" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="106" t="s">
         <v>119</v>
       </c>
-      <c r="B21" s="104"/>
-      <c r="C21" s="84" t="s">
+      <c r="B21" s="107"/>
+      <c r="C21" s="87" t="s">
         <v>198</v>
       </c>
-      <c r="D21" s="85"/>
-      <c r="E21" s="85"/>
-      <c r="F21" s="85"/>
-      <c r="G21" s="86"/>
+      <c r="D21" s="88"/>
+      <c r="E21" s="88"/>
+      <c r="F21" s="88"/>
+      <c r="G21" s="89"/>
       <c r="H21" s="69" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosAgenda</v>
       </c>
-      <c r="I21" s="109" t="str">
+      <c r="I21" s="112" t="str">
         <f>B2</f>
         <v>Agenda</v>
       </c>
-      <c r="J21" s="112" t="str">
+      <c r="J21" s="115" t="str">
         <f>_xlfn.CONCAT("Corresponde al objeto que internamente contiene los datos necesarios para crear una nueva ",$B$2,)</f>
         <v>Corresponde al objeto que internamente contiene los datos necesarios para crear una nueva Agenda</v>
       </c>
       <c r="K21" s="50"/>
-      <c r="L21" s="84"/>
-      <c r="M21" s="85"/>
-      <c r="N21" s="85"/>
-      <c r="O21" s="86"/>
+      <c r="L21" s="87"/>
+      <c r="M21" s="88"/>
+      <c r="N21" s="88"/>
+      <c r="O21" s="89"/>
       <c r="P21" s="14" t="s">
         <v>187</v>
       </c>
@@ -5253,22 +5257,22 @@
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="108.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="105"/>
-      <c r="B22" s="106"/>
-      <c r="C22" s="87"/>
-      <c r="D22" s="88"/>
-      <c r="E22" s="88"/>
-      <c r="F22" s="88"/>
-      <c r="G22" s="89"/>
+    <row r="22" spans="1:19" ht="108.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="108"/>
+      <c r="B22" s="109"/>
+      <c r="C22" s="90"/>
+      <c r="D22" s="91"/>
+      <c r="E22" s="91"/>
+      <c r="F22" s="91"/>
+      <c r="G22" s="92"/>
       <c r="H22" s="70"/>
-      <c r="I22" s="110"/>
-      <c r="J22" s="113"/>
+      <c r="I22" s="113"/>
+      <c r="J22" s="116"/>
       <c r="K22" s="52"/>
-      <c r="L22" s="87"/>
-      <c r="M22" s="88"/>
-      <c r="N22" s="88"/>
-      <c r="O22" s="89"/>
+      <c r="L22" s="90"/>
+      <c r="M22" s="91"/>
+      <c r="N22" s="91"/>
+      <c r="O22" s="92"/>
       <c r="P22" s="14" t="s">
         <v>188</v>
       </c>
@@ -5282,22 +5286,22 @@
         <v>122</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="123.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="105"/>
-      <c r="B23" s="106"/>
-      <c r="C23" s="87"/>
-      <c r="D23" s="88"/>
-      <c r="E23" s="88"/>
-      <c r="F23" s="88"/>
-      <c r="G23" s="89"/>
+    <row r="23" spans="1:19" ht="123.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="108"/>
+      <c r="B23" s="109"/>
+      <c r="C23" s="90"/>
+      <c r="D23" s="91"/>
+      <c r="E23" s="91"/>
+      <c r="F23" s="91"/>
+      <c r="G23" s="92"/>
       <c r="H23" s="70"/>
-      <c r="I23" s="110"/>
-      <c r="J23" s="113"/>
+      <c r="I23" s="113"/>
+      <c r="J23" s="116"/>
       <c r="K23" s="52"/>
-      <c r="L23" s="87"/>
-      <c r="M23" s="88"/>
-      <c r="N23" s="88"/>
-      <c r="O23" s="89"/>
+      <c r="L23" s="90"/>
+      <c r="M23" s="91"/>
+      <c r="N23" s="91"/>
+      <c r="O23" s="92"/>
       <c r="P23" s="14" t="s">
         <v>189</v>
       </c>
@@ -5311,22 +5315,22 @@
         <v>122</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="111" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="105"/>
-      <c r="B24" s="106"/>
-      <c r="C24" s="87"/>
-      <c r="D24" s="88"/>
-      <c r="E24" s="88"/>
-      <c r="F24" s="88"/>
-      <c r="G24" s="89"/>
+    <row r="24" spans="1:19" ht="111" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="108"/>
+      <c r="B24" s="109"/>
+      <c r="C24" s="90"/>
+      <c r="D24" s="91"/>
+      <c r="E24" s="91"/>
+      <c r="F24" s="91"/>
+      <c r="G24" s="92"/>
       <c r="H24" s="70"/>
-      <c r="I24" s="110"/>
-      <c r="J24" s="113"/>
+      <c r="I24" s="113"/>
+      <c r="J24" s="116"/>
       <c r="K24" s="52"/>
-      <c r="L24" s="87"/>
-      <c r="M24" s="88"/>
-      <c r="N24" s="88"/>
-      <c r="O24" s="89"/>
+      <c r="L24" s="90"/>
+      <c r="M24" s="91"/>
+      <c r="N24" s="91"/>
+      <c r="O24" s="92"/>
       <c r="P24" s="14" t="s">
         <v>190</v>
       </c>
@@ -5340,22 +5344,22 @@
         <v>205</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="87.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="107"/>
-      <c r="B25" s="108"/>
-      <c r="C25" s="90"/>
-      <c r="D25" s="91"/>
-      <c r="E25" s="91"/>
-      <c r="F25" s="91"/>
-      <c r="G25" s="92"/>
+    <row r="25" spans="1:19" ht="87.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="110"/>
+      <c r="B25" s="111"/>
+      <c r="C25" s="93"/>
+      <c r="D25" s="94"/>
+      <c r="E25" s="94"/>
+      <c r="F25" s="94"/>
+      <c r="G25" s="95"/>
       <c r="H25" s="71"/>
-      <c r="I25" s="111"/>
-      <c r="J25" s="114"/>
+      <c r="I25" s="114"/>
+      <c r="J25" s="117"/>
       <c r="K25" s="53"/>
-      <c r="L25" s="90"/>
-      <c r="M25" s="91"/>
-      <c r="N25" s="91"/>
-      <c r="O25" s="92"/>
+      <c r="L25" s="93"/>
+      <c r="M25" s="94"/>
+      <c r="N25" s="94"/>
+      <c r="O25" s="95"/>
       <c r="P25" s="14" t="s">
         <v>191</v>
       </c>
@@ -5369,18 +5373,18 @@
         <v>122</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="102.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="93" t="s">
+    <row r="26" spans="1:19" ht="102.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="96" t="s">
         <v>123</v>
       </c>
-      <c r="B26" s="94"/>
-      <c r="C26" s="95" t="s">
+      <c r="B26" s="97"/>
+      <c r="C26" s="98" t="s">
         <v>197</v>
       </c>
-      <c r="D26" s="95"/>
-      <c r="E26" s="95"/>
-      <c r="F26" s="95"/>
-      <c r="G26" s="95"/>
+      <c r="D26" s="98"/>
+      <c r="E26" s="98"/>
+      <c r="F26" s="98"/>
+      <c r="G26" s="98"/>
       <c r="H26" s="36" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosAgenda</v>
@@ -5396,12 +5400,12 @@
       <c r="K26" s="49" t="s">
         <v>124</v>
       </c>
-      <c r="L26" s="96" t="s">
+      <c r="L26" s="99" t="s">
         <v>201</v>
       </c>
-      <c r="M26" s="96"/>
-      <c r="N26" s="96"/>
-      <c r="O26" s="96"/>
+      <c r="M26" s="99"/>
+      <c r="N26" s="99"/>
+      <c r="O26" s="99"/>
       <c r="P26" s="23" t="s">
         <v>192</v>
       </c>
@@ -5415,18 +5419,18 @@
         <v>122</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A27" s="97" t="s">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A27" s="100" t="s">
         <v>127</v>
       </c>
-      <c r="B27" s="98"/>
-      <c r="C27" s="99" t="s">
+      <c r="B27" s="101"/>
+      <c r="C27" s="102" t="s">
         <v>199</v>
       </c>
-      <c r="D27" s="99"/>
-      <c r="E27" s="99"/>
-      <c r="F27" s="99"/>
-      <c r="G27" s="99"/>
+      <c r="D27" s="102"/>
+      <c r="E27" s="102"/>
+      <c r="F27" s="102"/>
+      <c r="G27" s="102"/>
       <c r="H27" s="39" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosAgenda</v>
@@ -5440,35 +5444,35 @@
         <v>Corresponde a los datos que se van a modificar de la Agenda</v>
       </c>
       <c r="K27" s="41"/>
-      <c r="L27" s="100"/>
-      <c r="M27" s="101"/>
-      <c r="N27" s="101"/>
-      <c r="O27" s="102"/>
-      <c r="P27" s="72" t="s">
+      <c r="L27" s="103"/>
+      <c r="M27" s="104"/>
+      <c r="N27" s="104"/>
+      <c r="O27" s="105"/>
+      <c r="P27" s="118" t="s">
         <v>193</v>
       </c>
-      <c r="Q27" s="74" t="s">
+      <c r="Q27" s="120" t="s">
         <v>130</v>
       </c>
-      <c r="R27" s="74" t="s">
+      <c r="R27" s="120" t="s">
         <v>131</v>
       </c>
-      <c r="S27" s="76" t="s">
+      <c r="S27" s="122" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="90.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="78" t="s">
+    <row r="28" spans="1:19" ht="90.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="124" t="s">
         <v>133</v>
       </c>
-      <c r="B28" s="79"/>
-      <c r="C28" s="80" t="s">
+      <c r="B28" s="125"/>
+      <c r="C28" s="126" t="s">
         <v>200</v>
       </c>
-      <c r="D28" s="80"/>
-      <c r="E28" s="80"/>
-      <c r="F28" s="80"/>
-      <c r="G28" s="80"/>
+      <c r="D28" s="126"/>
+      <c r="E28" s="126"/>
+      <c r="F28" s="126"/>
+      <c r="G28" s="126"/>
       <c r="H28" s="55" t="s">
         <v>46</v>
       </c>
@@ -5480,23 +5484,30 @@
         <v>Corresponde al identificador de la Agenda  que se quiere dar de baja.</v>
       </c>
       <c r="K28" s="43"/>
-      <c r="L28" s="81"/>
-      <c r="M28" s="82"/>
-      <c r="N28" s="82"/>
-      <c r="O28" s="83"/>
-      <c r="P28" s="73"/>
-      <c r="Q28" s="75"/>
-      <c r="R28" s="75"/>
-      <c r="S28" s="77"/>
+      <c r="L28" s="127"/>
+      <c r="M28" s="128"/>
+      <c r="N28" s="128"/>
+      <c r="O28" s="129"/>
+      <c r="P28" s="119"/>
+      <c r="Q28" s="121"/>
+      <c r="R28" s="121"/>
+      <c r="S28" s="123"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="L21:O25"/>
-    <mergeCell ref="A21:B25"/>
-    <mergeCell ref="C21:G25"/>
-    <mergeCell ref="H21:H25"/>
-    <mergeCell ref="I21:I25"/>
-    <mergeCell ref="J21:J25"/>
+    <mergeCell ref="R27:R28"/>
+    <mergeCell ref="S27:S28"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="L28:O28"/>
+    <mergeCell ref="P27:P28"/>
+    <mergeCell ref="Q27:Q28"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="L26:O26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="L27:O27"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="L20:O20"/>
     <mergeCell ref="A1:Q1"/>
@@ -5511,19 +5522,12 @@
     <mergeCell ref="K19:O19"/>
     <mergeCell ref="P19:Q19"/>
     <mergeCell ref="C14:C15"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="L26:O26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="L27:O27"/>
-    <mergeCell ref="R27:R28"/>
-    <mergeCell ref="S27:S28"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="L28:O28"/>
-    <mergeCell ref="P27:P28"/>
-    <mergeCell ref="Q27:Q28"/>
+    <mergeCell ref="L21:O25"/>
+    <mergeCell ref="A21:B25"/>
+    <mergeCell ref="C21:G25"/>
+    <mergeCell ref="H21:H25"/>
+    <mergeCell ref="I21:I25"/>
+    <mergeCell ref="J21:J25"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de Dominio'!A1" display="Volver al inicio" xr:uid="{B2E38F92-070F-4A08-9587-748CDC5E3622}"/>
@@ -5554,103 +5558,103 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC57795F-B02D-497B-A04E-44BC1D3D4128}">
   <dimension ref="A1:U27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5546875" style="8" customWidth="1"/>
-    <col min="3" max="3" width="25.88671875" style="8" customWidth="1"/>
-    <col min="4" max="4" width="18.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="61.33203125" style="8" customWidth="1"/>
-    <col min="10" max="10" width="79.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="25.85546875" style="8" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="61.28515625" style="8" customWidth="1"/>
+    <col min="10" max="10" width="79.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.85546875" style="8" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="25" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="94.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="132.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="46.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="50.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="66.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="52.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="11.44140625" style="8"/>
+    <col min="17" max="17" width="94.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="132.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="46.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="50.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="66.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="52.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="11.42578125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A1" s="121" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A1" s="78" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
-      <c r="F1" s="121"/>
-      <c r="G1" s="121"/>
-      <c r="H1" s="121"/>
-      <c r="I1" s="121"/>
-      <c r="J1" s="121"/>
-      <c r="K1" s="121"/>
-      <c r="L1" s="121"/>
-      <c r="M1" s="121"/>
-      <c r="N1" s="121"/>
-      <c r="O1" s="121"/>
-      <c r="P1" s="121"/>
-      <c r="Q1" s="121"/>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
+      <c r="P1" s="78"/>
+      <c r="Q1" s="78"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="122" t="str">
+      <c r="B2" s="79" t="str">
         <f>'Listado Objetos de Dominio'!A5</f>
         <v>Turno</v>
       </c>
-      <c r="C2" s="122"/>
-      <c r="D2" s="122"/>
-      <c r="E2" s="122"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="122"/>
-      <c r="H2" s="122"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="122"/>
-      <c r="K2" s="122"/>
-      <c r="L2" s="122"/>
-      <c r="M2" s="122"/>
-      <c r="N2" s="122"/>
-      <c r="O2" s="122"/>
-      <c r="P2" s="122"/>
-      <c r="Q2" s="122"/>
-    </row>
-    <row r="3" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="79"/>
+      <c r="M2" s="79"/>
+      <c r="N2" s="79"/>
+      <c r="O2" s="79"/>
+      <c r="P2" s="79"/>
+      <c r="Q2" s="79"/>
+    </row>
+    <row r="3" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="123" t="str">
+      <c r="B3" s="80" t="str">
         <f>'Listado Objetos de Dominio'!B5</f>
         <v>Objeto de dominio que representa uno de los turnos que representan un bloque de tiempo que el residente podrá reservar.</v>
       </c>
-      <c r="C3" s="123"/>
-      <c r="D3" s="123"/>
-      <c r="E3" s="123"/>
-      <c r="F3" s="123"/>
-      <c r="G3" s="123"/>
-      <c r="H3" s="123"/>
-      <c r="I3" s="123"/>
-      <c r="J3" s="123"/>
-      <c r="K3" s="123"/>
-      <c r="L3" s="123"/>
-      <c r="M3" s="123"/>
-      <c r="N3" s="123"/>
-      <c r="O3" s="123"/>
-      <c r="P3" s="123"/>
-      <c r="Q3" s="123"/>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="80"/>
+      <c r="L3" s="80"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="80"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="80"/>
+      <c r="Q3" s="80"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>30</v>
       </c>
@@ -5719,7 +5723,7 @@
         <v>Eliminar</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
         <v>46</v>
       </c>
@@ -5772,7 +5776,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
         <v>109</v>
       </c>
@@ -5827,7 +5831,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
         <v>83</v>
       </c>
@@ -5876,7 +5880,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
         <v>84</v>
       </c>
@@ -5925,7 +5929,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
         <v>110</v>
       </c>
@@ -5974,7 +5978,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="48" t="s">
         <v>85</v>
       </c>
@@ -6021,15 +6025,15 @@
         <v>140</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="12" spans="1:21" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="118" t="s">
+    <row r="11" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="75" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="119"/>
-      <c r="C12" s="120"/>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B12" s="76"/>
+      <c r="C12" s="77"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
         <v>53</v>
       </c>
@@ -6040,80 +6044,80 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="130" t="s">
         <v>118</v>
       </c>
-      <c r="B14" s="126" t="s">
+      <c r="B14" s="83" t="s">
         <v>117</v>
       </c>
       <c r="C14" s="30" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="131"/>
       <c r="B15" s="133"/>
       <c r="C15" s="30" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="131"/>
       <c r="B16" s="133"/>
       <c r="C16" s="30" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:19" ht="20.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="132"/>
-      <c r="B17" s="127"/>
+      <c r="B17" s="84"/>
       <c r="C17" s="46" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A19" s="128" t="s">
+    <row r="18" spans="1:19" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A19" s="85" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="115"/>
-      <c r="C19" s="115" t="s">
+      <c r="B19" s="72"/>
+      <c r="C19" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="115"/>
-      <c r="E19" s="115"/>
-      <c r="F19" s="115"/>
-      <c r="G19" s="115"/>
-      <c r="H19" s="115" t="s">
+      <c r="D19" s="72"/>
+      <c r="E19" s="72"/>
+      <c r="F19" s="72"/>
+      <c r="G19" s="72"/>
+      <c r="H19" s="72" t="s">
         <v>56</v>
       </c>
-      <c r="I19" s="115"/>
-      <c r="J19" s="115"/>
-      <c r="K19" s="115" t="s">
+      <c r="I19" s="72"/>
+      <c r="J19" s="72"/>
+      <c r="K19" s="72" t="s">
         <v>57</v>
       </c>
-      <c r="L19" s="115"/>
-      <c r="M19" s="115"/>
-      <c r="N19" s="115"/>
-      <c r="O19" s="115"/>
-      <c r="P19" s="115" t="s">
+      <c r="L19" s="72"/>
+      <c r="M19" s="72"/>
+      <c r="N19" s="72"/>
+      <c r="O19" s="72"/>
+      <c r="P19" s="72" t="s">
         <v>58</v>
       </c>
-      <c r="Q19" s="115"/>
-      <c r="R19" s="115" t="s">
+      <c r="Q19" s="72"/>
+      <c r="R19" s="72" t="s">
         <v>59</v>
       </c>
-      <c r="S19" s="116"/>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A20" s="129"/>
-      <c r="B20" s="117"/>
-      <c r="C20" s="117"/>
-      <c r="D20" s="117"/>
-      <c r="E20" s="117"/>
-      <c r="F20" s="117"/>
-      <c r="G20" s="117"/>
+      <c r="S19" s="73"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20" s="86"/>
+      <c r="B20" s="74"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="74"/>
+      <c r="E20" s="74"/>
+      <c r="F20" s="74"/>
+      <c r="G20" s="74"/>
       <c r="H20" s="32" t="s">
         <v>60</v>
       </c>
@@ -6126,12 +6130,12 @@
       <c r="K20" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="L20" s="117" t="s">
+      <c r="L20" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="M20" s="117"/>
-      <c r="N20" s="117"/>
-      <c r="O20" s="117"/>
+      <c r="M20" s="74"/>
+      <c r="N20" s="74"/>
+      <c r="O20" s="74"/>
       <c r="P20" s="32" t="s">
         <v>62</v>
       </c>
@@ -6145,35 +6149,35 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="151.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="103" t="s">
+    <row r="21" spans="1:19" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="106" t="s">
         <v>119</v>
       </c>
-      <c r="B21" s="104"/>
-      <c r="C21" s="84" t="s">
+      <c r="B21" s="107"/>
+      <c r="C21" s="87" t="s">
         <v>173</v>
       </c>
-      <c r="D21" s="85"/>
-      <c r="E21" s="85"/>
-      <c r="F21" s="85"/>
-      <c r="G21" s="86"/>
+      <c r="D21" s="88"/>
+      <c r="E21" s="88"/>
+      <c r="F21" s="88"/>
+      <c r="G21" s="89"/>
       <c r="H21" s="69" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosTurno</v>
       </c>
-      <c r="I21" s="109" t="str">
+      <c r="I21" s="112" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosTurno</v>
       </c>
-      <c r="J21" s="112" t="str">
+      <c r="J21" s="115" t="str">
         <f>_xlfn.CONCAT("Corresponde al objeto que internamente contiene los datos necesarios para crear una nueva ",$B$2,)</f>
         <v>Corresponde al objeto que internamente contiene los datos necesarios para crear una nueva Turno</v>
       </c>
       <c r="K21" s="50"/>
-      <c r="L21" s="84"/>
-      <c r="M21" s="85"/>
-      <c r="N21" s="85"/>
-      <c r="O21" s="86"/>
+      <c r="L21" s="87"/>
+      <c r="M21" s="88"/>
+      <c r="N21" s="88"/>
+      <c r="O21" s="89"/>
       <c r="P21" s="14" t="s">
         <v>165</v>
       </c>
@@ -6187,22 +6191,22 @@
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="151.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="105"/>
-      <c r="B22" s="106"/>
-      <c r="C22" s="87"/>
-      <c r="D22" s="88"/>
-      <c r="E22" s="88"/>
-      <c r="F22" s="88"/>
-      <c r="G22" s="89"/>
+    <row r="22" spans="1:19" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="108"/>
+      <c r="B22" s="109"/>
+      <c r="C22" s="90"/>
+      <c r="D22" s="91"/>
+      <c r="E22" s="91"/>
+      <c r="F22" s="91"/>
+      <c r="G22" s="92"/>
       <c r="H22" s="70"/>
-      <c r="I22" s="110"/>
-      <c r="J22" s="113"/>
+      <c r="I22" s="113"/>
+      <c r="J22" s="116"/>
       <c r="K22" s="52"/>
-      <c r="L22" s="87"/>
-      <c r="M22" s="88"/>
-      <c r="N22" s="88"/>
-      <c r="O22" s="89"/>
+      <c r="L22" s="90"/>
+      <c r="M22" s="91"/>
+      <c r="N22" s="91"/>
+      <c r="O22" s="92"/>
       <c r="P22" s="14" t="s">
         <v>166</v>
       </c>
@@ -6216,22 +6220,22 @@
         <v>178</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="75.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="105"/>
-      <c r="B23" s="106"/>
-      <c r="C23" s="87"/>
-      <c r="D23" s="88"/>
-      <c r="E23" s="88"/>
-      <c r="F23" s="88"/>
-      <c r="G23" s="89"/>
+    <row r="23" spans="1:19" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="108"/>
+      <c r="B23" s="109"/>
+      <c r="C23" s="90"/>
+      <c r="D23" s="91"/>
+      <c r="E23" s="91"/>
+      <c r="F23" s="91"/>
+      <c r="G23" s="92"/>
       <c r="H23" s="70"/>
-      <c r="I23" s="110"/>
-      <c r="J23" s="113"/>
+      <c r="I23" s="113"/>
+      <c r="J23" s="116"/>
       <c r="K23" s="52"/>
-      <c r="L23" s="87"/>
-      <c r="M23" s="88"/>
-      <c r="N23" s="88"/>
-      <c r="O23" s="89"/>
+      <c r="L23" s="90"/>
+      <c r="M23" s="91"/>
+      <c r="N23" s="91"/>
+      <c r="O23" s="92"/>
       <c r="P23" s="14" t="s">
         <v>167</v>
       </c>
@@ -6245,22 +6249,22 @@
         <v>178</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="77.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="107"/>
-      <c r="B24" s="108"/>
-      <c r="C24" s="90"/>
-      <c r="D24" s="91"/>
-      <c r="E24" s="91"/>
-      <c r="F24" s="91"/>
-      <c r="G24" s="92"/>
+    <row r="24" spans="1:19" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="110"/>
+      <c r="B24" s="111"/>
+      <c r="C24" s="93"/>
+      <c r="D24" s="94"/>
+      <c r="E24" s="94"/>
+      <c r="F24" s="94"/>
+      <c r="G24" s="95"/>
       <c r="H24" s="71"/>
-      <c r="I24" s="111"/>
-      <c r="J24" s="114"/>
+      <c r="I24" s="114"/>
+      <c r="J24" s="117"/>
       <c r="K24" s="53"/>
-      <c r="L24" s="90"/>
-      <c r="M24" s="91"/>
-      <c r="N24" s="91"/>
-      <c r="O24" s="92"/>
+      <c r="L24" s="93"/>
+      <c r="M24" s="94"/>
+      <c r="N24" s="94"/>
+      <c r="O24" s="95"/>
       <c r="P24" s="14" t="s">
         <v>168</v>
       </c>
@@ -6274,18 +6278,18 @@
         <v>181</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="105" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="93" t="s">
+    <row r="25" spans="1:19" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="96" t="s">
         <v>123</v>
       </c>
-      <c r="B25" s="94"/>
-      <c r="C25" s="95" t="s">
+      <c r="B25" s="97"/>
+      <c r="C25" s="98" t="s">
         <v>176</v>
       </c>
-      <c r="D25" s="95"/>
-      <c r="E25" s="95"/>
-      <c r="F25" s="95"/>
-      <c r="G25" s="95"/>
+      <c r="D25" s="98"/>
+      <c r="E25" s="98"/>
+      <c r="F25" s="98"/>
+      <c r="G25" s="98"/>
       <c r="H25" s="36" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosTurno</v>
@@ -6301,12 +6305,12 @@
       <c r="K25" s="49" t="s">
         <v>124</v>
       </c>
-      <c r="L25" s="96" t="s">
+      <c r="L25" s="99" t="s">
         <v>182</v>
       </c>
-      <c r="M25" s="96"/>
-      <c r="N25" s="96"/>
-      <c r="O25" s="96"/>
+      <c r="M25" s="99"/>
+      <c r="N25" s="99"/>
+      <c r="O25" s="99"/>
       <c r="P25" s="23" t="s">
         <v>183</v>
       </c>
@@ -6320,18 +6324,18 @@
         <v>122</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="97" t="s">
+    <row r="26" spans="1:19" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="100" t="s">
         <v>127</v>
       </c>
-      <c r="B26" s="98"/>
-      <c r="C26" s="99" t="s">
+      <c r="B26" s="101"/>
+      <c r="C26" s="102" t="s">
         <v>174</v>
       </c>
-      <c r="D26" s="99"/>
-      <c r="E26" s="99"/>
-      <c r="F26" s="99"/>
-      <c r="G26" s="99"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="102"/>
+      <c r="F26" s="102"/>
+      <c r="G26" s="102"/>
       <c r="H26" s="39" t="str">
         <f>_xlfn.CONCAT("datos",$B$2)</f>
         <v>datosTurno</v>
@@ -6345,10 +6349,10 @@
         <v>Corresponde a los datos que se van a modificar de la Turno</v>
       </c>
       <c r="K26" s="41"/>
-      <c r="L26" s="100"/>
-      <c r="M26" s="101"/>
-      <c r="N26" s="101"/>
-      <c r="O26" s="102"/>
+      <c r="L26" s="103"/>
+      <c r="M26" s="104"/>
+      <c r="N26" s="104"/>
+      <c r="O26" s="105"/>
       <c r="P26" s="62" t="s">
         <v>184</v>
       </c>
@@ -6362,18 +6366,18 @@
         <v>132</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="84.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="78" t="s">
+    <row r="27" spans="1:19" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="124" t="s">
         <v>133</v>
       </c>
-      <c r="B27" s="79"/>
-      <c r="C27" s="80" t="s">
+      <c r="B27" s="125"/>
+      <c r="C27" s="126" t="s">
         <v>175</v>
       </c>
-      <c r="D27" s="80"/>
-      <c r="E27" s="80"/>
-      <c r="F27" s="80"/>
-      <c r="G27" s="80"/>
+      <c r="D27" s="126"/>
+      <c r="E27" s="126"/>
+      <c r="F27" s="126"/>
+      <c r="G27" s="126"/>
       <c r="H27" s="55" t="s">
         <v>46</v>
       </c>
@@ -6385,10 +6389,10 @@
         <v>Corresponde al identificador de la Turno  que se quiere dar de baja.</v>
       </c>
       <c r="K27" s="43"/>
-      <c r="L27" s="81"/>
-      <c r="M27" s="82"/>
-      <c r="N27" s="82"/>
-      <c r="O27" s="83"/>
+      <c r="L27" s="127"/>
+      <c r="M27" s="128"/>
+      <c r="N27" s="128"/>
+      <c r="O27" s="129"/>
       <c r="P27" s="44" t="s">
         <v>184</v>
       </c>
@@ -6404,12 +6408,15 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="L21:O24"/>
-    <mergeCell ref="A21:B24"/>
-    <mergeCell ref="C21:G24"/>
-    <mergeCell ref="H21:H24"/>
-    <mergeCell ref="I21:I24"/>
-    <mergeCell ref="J21:J24"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="L27:O27"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="L25:O25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="L26:O26"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="L20:O20"/>
     <mergeCell ref="A1:Q1"/>
@@ -6423,15 +6430,12 @@
     <mergeCell ref="H19:J19"/>
     <mergeCell ref="K19:O19"/>
     <mergeCell ref="P19:Q19"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="L27:O27"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="L25:O25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="L26:O26"/>
+    <mergeCell ref="L21:O24"/>
+    <mergeCell ref="A21:B24"/>
+    <mergeCell ref="C21:G24"/>
+    <mergeCell ref="H21:H24"/>
+    <mergeCell ref="I21:I24"/>
+    <mergeCell ref="J21:J24"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de Dominio'!A1" display="Volver al inicio" xr:uid="{186E73A2-C89F-4A82-8727-EBDE505719F2}"/>

</xml_diff>